<commit_message>
:sparkles: add Passive smoker code to SmokingStatus value set
</commit_message>
<xml_diff>
--- a/CommonDataModel.xlsx
+++ b/CommonDataModel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\doguk\OneDrive\Desktop\DT4H\Repositories\common-data-model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\db\dt4h\common-data-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EBE9FB-1E54-4893-AAB1-CBABD7E21BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAC1BCF-B7D7-4289-BB41-6339F2BD48B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="901" firstSheet="12" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="10635" windowWidth="38640" windowHeight="21120" tabRatio="901" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="10" r:id="rId1"/>
@@ -864,7 +864,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4694" uniqueCount="2025">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4696" uniqueCount="2026">
   <si>
     <t>Required</t>
   </si>
@@ -6959,6 +6959,9 @@
   </si>
   <si>
     <t>Anti diabetics</t>
+  </si>
+  <si>
+    <t>Passive smoker</t>
   </si>
 </sst>
 </file>
@@ -7337,22 +7340,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8340,7 +8343,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1770B9A2-CDA6-4E37-82EC-A9C07EE24319}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.5546875" customWidth="1"/>
@@ -8710,15 +8713,21 @@
       <c r="H20" s="66"/>
       <c r="I20" s="66"/>
     </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>2025</v>
+      </c>
+      <c r="B21" s="51">
+        <v>43381005</v>
+      </c>
+      <c r="C21" s="65" t="s">
+        <v>158</v>
+      </c>
+      <c r="D21" s="65"/>
+    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:I14"/>
+  <mergeCells count="18">
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="C20:D20"/>
@@ -8729,6 +8738,13 @@
     <mergeCell ref="F17:I17"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:I14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9587,41 +9603,14 @@
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F38:I38"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C41:D41"/>
@@ -9638,14 +9627,41 @@
     <mergeCell ref="F31:I31"/>
     <mergeCell ref="F32:I32"/>
     <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:I14"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E13:E41" xr:uid="{14C408A9-075A-4B77-84C3-9F689D082B68}">
@@ -10345,13 +10361,13 @@
         <v>462</v>
       </c>
       <c r="D39" s="67"/>
-      <c r="E39" s="71"/>
-      <c r="F39" s="72" t="s">
+      <c r="E39" s="70"/>
+      <c r="F39" s="73" t="s">
         <v>463</v>
       </c>
-      <c r="G39" s="72"/>
-      <c r="H39" s="72"/>
-      <c r="I39" s="72"/>
+      <c r="G39" s="73"/>
+      <c r="H39" s="73"/>
+      <c r="I39" s="73"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="42" t="s">
@@ -10360,11 +10376,11 @@
       <c r="B40" s="42" t="s">
         <v>465</v>
       </c>
-      <c r="C40" s="69" t="s">
+      <c r="C40" s="71" t="s">
         <v>466</v>
       </c>
-      <c r="D40" s="69"/>
-      <c r="E40" s="70"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="72"/>
       <c r="F40" s="68"/>
       <c r="G40" s="66"/>
       <c r="H40" s="66"/>
@@ -10377,11 +10393,11 @@
       <c r="B41" s="42" t="s">
         <v>468</v>
       </c>
-      <c r="C41" s="69" t="s">
+      <c r="C41" s="71" t="s">
         <v>469</v>
       </c>
-      <c r="D41" s="69"/>
-      <c r="E41" s="70"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="72"/>
       <c r="F41" s="68"/>
       <c r="G41" s="66"/>
       <c r="H41" s="66"/>
@@ -10394,11 +10410,11 @@
       <c r="B42" s="42" t="s">
         <v>471</v>
       </c>
-      <c r="C42" s="69" t="s">
+      <c r="C42" s="71" t="s">
         <v>472</v>
       </c>
-      <c r="D42" s="69"/>
-      <c r="E42" s="70"/>
+      <c r="D42" s="71"/>
+      <c r="E42" s="72"/>
       <c r="F42" s="68"/>
       <c r="G42" s="66"/>
       <c r="H42" s="66"/>
@@ -10411,11 +10427,11 @@
       <c r="B43" s="42" t="s">
         <v>474</v>
       </c>
-      <c r="C43" s="69" t="s">
+      <c r="C43" s="71" t="s">
         <v>2012</v>
       </c>
-      <c r="D43" s="69"/>
-      <c r="E43" s="70"/>
+      <c r="D43" s="71"/>
+      <c r="E43" s="72"/>
       <c r="F43" s="68"/>
       <c r="G43" s="66"/>
       <c r="H43" s="66"/>
@@ -10428,11 +10444,11 @@
       <c r="B44" s="42" t="s">
         <v>476</v>
       </c>
-      <c r="C44" s="69" t="s">
+      <c r="C44" s="71" t="s">
         <v>477</v>
       </c>
-      <c r="D44" s="69"/>
-      <c r="E44" s="70"/>
+      <c r="D44" s="71"/>
+      <c r="E44" s="72"/>
       <c r="F44" s="68"/>
       <c r="G44" s="66"/>
       <c r="H44" s="66"/>
@@ -10445,11 +10461,11 @@
       <c r="B45" s="42" t="s">
         <v>479</v>
       </c>
-      <c r="C45" s="69" t="s">
+      <c r="C45" s="71" t="s">
         <v>480</v>
       </c>
-      <c r="D45" s="69"/>
-      <c r="E45" s="70"/>
+      <c r="D45" s="71"/>
+      <c r="E45" s="72"/>
       <c r="F45" s="68"/>
       <c r="G45" s="66"/>
       <c r="H45" s="66"/>
@@ -10462,11 +10478,11 @@
       <c r="B46" s="42" t="s">
         <v>482</v>
       </c>
-      <c r="C46" s="69" t="s">
+      <c r="C46" s="71" t="s">
         <v>483</v>
       </c>
-      <c r="D46" s="69"/>
-      <c r="E46" s="70"/>
+      <c r="D46" s="71"/>
+      <c r="E46" s="72"/>
       <c r="F46" s="68"/>
       <c r="G46" s="66"/>
       <c r="H46" s="66"/>
@@ -10479,11 +10495,11 @@
       <c r="B47" s="42" t="s">
         <v>485</v>
       </c>
-      <c r="C47" s="69" t="s">
+      <c r="C47" s="71" t="s">
         <v>2022</v>
       </c>
-      <c r="D47" s="69"/>
-      <c r="E47" s="70"/>
+      <c r="D47" s="71"/>
+      <c r="E47" s="72"/>
       <c r="F47" s="68"/>
       <c r="G47" s="66"/>
       <c r="H47" s="66"/>
@@ -10496,11 +10512,11 @@
       <c r="B48" s="42" t="s">
         <v>486</v>
       </c>
-      <c r="C48" s="69" t="s">
+      <c r="C48" s="71" t="s">
         <v>2013</v>
       </c>
-      <c r="D48" s="69"/>
-      <c r="E48" s="70"/>
+      <c r="D48" s="71"/>
+      <c r="E48" s="72"/>
       <c r="F48" s="68"/>
       <c r="G48" s="66"/>
       <c r="H48" s="66"/>
@@ -10513,11 +10529,11 @@
       <c r="B49" s="42" t="s">
         <v>488</v>
       </c>
-      <c r="C49" s="69" t="s">
+      <c r="C49" s="71" t="s">
         <v>489</v>
       </c>
-      <c r="D49" s="69"/>
-      <c r="E49" s="70"/>
+      <c r="D49" s="71"/>
+      <c r="E49" s="72"/>
       <c r="F49" s="68"/>
       <c r="G49" s="66"/>
       <c r="H49" s="66"/>
@@ -10530,11 +10546,11 @@
       <c r="B50" s="42" t="s">
         <v>491</v>
       </c>
-      <c r="C50" s="69" t="s">
+      <c r="C50" s="71" t="s">
         <v>492</v>
       </c>
-      <c r="D50" s="69"/>
-      <c r="E50" s="70"/>
+      <c r="D50" s="71"/>
+      <c r="E50" s="72"/>
       <c r="F50" s="68"/>
       <c r="G50" s="66"/>
       <c r="H50" s="66"/>
@@ -10547,11 +10563,11 @@
       <c r="B51" s="42" t="s">
         <v>494</v>
       </c>
-      <c r="C51" s="69" t="s">
+      <c r="C51" s="71" t="s">
         <v>495</v>
       </c>
-      <c r="D51" s="69"/>
-      <c r="E51" s="70"/>
+      <c r="D51" s="71"/>
+      <c r="E51" s="72"/>
       <c r="F51" s="68"/>
       <c r="G51" s="66"/>
       <c r="H51" s="66"/>
@@ -10564,11 +10580,11 @@
       <c r="B52" s="42" t="s">
         <v>497</v>
       </c>
-      <c r="C52" s="69" t="s">
+      <c r="C52" s="71" t="s">
         <v>498</v>
       </c>
-      <c r="D52" s="69"/>
-      <c r="E52" s="70"/>
+      <c r="D52" s="71"/>
+      <c r="E52" s="72"/>
       <c r="F52" s="68"/>
       <c r="G52" s="66"/>
       <c r="H52" s="66"/>
@@ -10581,11 +10597,11 @@
       <c r="B53" s="42" t="s">
         <v>500</v>
       </c>
-      <c r="C53" s="69" t="s">
+      <c r="C53" s="71" t="s">
         <v>501</v>
       </c>
-      <c r="D53" s="69"/>
-      <c r="E53" s="70"/>
+      <c r="D53" s="71"/>
+      <c r="E53" s="72"/>
       <c r="F53" s="68"/>
       <c r="G53" s="66"/>
       <c r="H53" s="66"/>
@@ -10598,11 +10614,11 @@
       <c r="B54" s="42" t="s">
         <v>503</v>
       </c>
-      <c r="C54" s="69" t="s">
+      <c r="C54" s="71" t="s">
         <v>504</v>
       </c>
-      <c r="D54" s="69"/>
-      <c r="E54" s="70"/>
+      <c r="D54" s="71"/>
+      <c r="E54" s="72"/>
       <c r="F54" s="68"/>
       <c r="G54" s="66"/>
       <c r="H54" s="66"/>
@@ -10615,11 +10631,11 @@
       <c r="B55" s="42" t="s">
         <v>506</v>
       </c>
-      <c r="C55" s="69" t="s">
+      <c r="C55" s="71" t="s">
         <v>507</v>
       </c>
-      <c r="D55" s="69"/>
-      <c r="E55" s="70"/>
+      <c r="D55" s="71"/>
+      <c r="E55" s="72"/>
       <c r="F55" s="68"/>
       <c r="G55" s="66"/>
       <c r="H55" s="66"/>
@@ -10632,11 +10648,11 @@
       <c r="B56" s="42" t="s">
         <v>509</v>
       </c>
-      <c r="C56" s="69" t="s">
+      <c r="C56" s="71" t="s">
         <v>510</v>
       </c>
-      <c r="D56" s="69"/>
-      <c r="E56" s="70"/>
+      <c r="D56" s="71"/>
+      <c r="E56" s="72"/>
       <c r="F56" s="68"/>
       <c r="G56" s="66"/>
       <c r="H56" s="66"/>
@@ -10649,11 +10665,11 @@
       <c r="B57" s="42" t="s">
         <v>512</v>
       </c>
-      <c r="C57" s="69" t="s">
+      <c r="C57" s="71" t="s">
         <v>513</v>
       </c>
-      <c r="D57" s="69"/>
-      <c r="E57" s="70"/>
+      <c r="D57" s="71"/>
+      <c r="E57" s="72"/>
       <c r="F57" s="68"/>
       <c r="G57" s="66"/>
       <c r="H57" s="66"/>
@@ -10666,11 +10682,11 @@
       <c r="B58" s="42" t="s">
         <v>515</v>
       </c>
-      <c r="C58" s="69" t="s">
+      <c r="C58" s="71" t="s">
         <v>516</v>
       </c>
-      <c r="D58" s="69"/>
-      <c r="E58" s="70"/>
+      <c r="D58" s="71"/>
+      <c r="E58" s="72"/>
       <c r="F58" s="68"/>
       <c r="G58" s="66"/>
       <c r="H58" s="66"/>
@@ -10683,11 +10699,11 @@
       <c r="B59" s="42" t="s">
         <v>518</v>
       </c>
-      <c r="C59" s="69" t="s">
+      <c r="C59" s="71" t="s">
         <v>519</v>
       </c>
-      <c r="D59" s="69"/>
-      <c r="E59" s="70"/>
+      <c r="D59" s="71"/>
+      <c r="E59" s="72"/>
       <c r="F59" s="68"/>
       <c r="G59" s="66"/>
       <c r="H59" s="66"/>
@@ -10700,11 +10716,11 @@
       <c r="B60" s="42" t="s">
         <v>521</v>
       </c>
-      <c r="C60" s="69" t="s">
+      <c r="C60" s="71" t="s">
         <v>522</v>
       </c>
-      <c r="D60" s="69"/>
-      <c r="E60" s="70"/>
+      <c r="D60" s="71"/>
+      <c r="E60" s="72"/>
       <c r="F60" s="68"/>
       <c r="G60" s="66"/>
       <c r="H60" s="66"/>
@@ -10717,11 +10733,11 @@
       <c r="B61" s="42" t="s">
         <v>524</v>
       </c>
-      <c r="C61" s="69" t="s">
+      <c r="C61" s="71" t="s">
         <v>525</v>
       </c>
-      <c r="D61" s="69"/>
-      <c r="E61" s="70"/>
+      <c r="D61" s="71"/>
+      <c r="E61" s="72"/>
       <c r="F61" s="68"/>
       <c r="G61" s="66"/>
       <c r="H61" s="66"/>
@@ -10734,11 +10750,11 @@
       <c r="B62" s="42" t="s">
         <v>527</v>
       </c>
-      <c r="C62" s="69" t="s">
+      <c r="C62" s="71" t="s">
         <v>528</v>
       </c>
-      <c r="D62" s="69"/>
-      <c r="E62" s="70"/>
+      <c r="D62" s="71"/>
+      <c r="E62" s="72"/>
       <c r="F62" s="68"/>
       <c r="G62" s="66"/>
       <c r="H62" s="66"/>
@@ -10751,11 +10767,11 @@
       <c r="B63" s="42" t="s">
         <v>530</v>
       </c>
-      <c r="C63" s="69" t="s">
+      <c r="C63" s="71" t="s">
         <v>531</v>
       </c>
-      <c r="D63" s="69"/>
-      <c r="E63" s="70"/>
+      <c r="D63" s="71"/>
+      <c r="E63" s="72"/>
       <c r="F63" s="68"/>
       <c r="G63" s="66"/>
       <c r="H63" s="66"/>
@@ -10768,11 +10784,11 @@
       <c r="B64" s="42" t="s">
         <v>532</v>
       </c>
-      <c r="C64" s="69" t="s">
+      <c r="C64" s="71" t="s">
         <v>533</v>
       </c>
-      <c r="D64" s="69"/>
-      <c r="E64" s="70"/>
+      <c r="D64" s="71"/>
+      <c r="E64" s="72"/>
       <c r="F64" s="68"/>
       <c r="G64" s="66"/>
       <c r="H64" s="66"/>
@@ -10785,11 +10801,11 @@
       <c r="B65" s="42" t="s">
         <v>535</v>
       </c>
-      <c r="C65" s="69" t="s">
+      <c r="C65" s="71" t="s">
         <v>536</v>
       </c>
-      <c r="D65" s="69"/>
-      <c r="E65" s="70"/>
+      <c r="D65" s="71"/>
+      <c r="E65" s="72"/>
       <c r="F65" s="68"/>
       <c r="G65" s="66"/>
       <c r="H65" s="66"/>
@@ -10802,11 +10818,11 @@
       <c r="B66" s="42" t="s">
         <v>538</v>
       </c>
-      <c r="C66" s="69" t="s">
+      <c r="C66" s="71" t="s">
         <v>2014</v>
       </c>
-      <c r="D66" s="69"/>
-      <c r="E66" s="70"/>
+      <c r="D66" s="71"/>
+      <c r="E66" s="72"/>
       <c r="F66" s="68"/>
       <c r="G66" s="66"/>
       <c r="H66" s="66"/>
@@ -10819,11 +10835,11 @@
       <c r="B67" s="42" t="s">
         <v>540</v>
       </c>
-      <c r="C67" s="69" t="s">
+      <c r="C67" s="71" t="s">
         <v>541</v>
       </c>
-      <c r="D67" s="69"/>
-      <c r="E67" s="70"/>
+      <c r="D67" s="71"/>
+      <c r="E67" s="72"/>
       <c r="F67" s="68"/>
       <c r="G67" s="66"/>
       <c r="H67" s="66"/>
@@ -10836,11 +10852,11 @@
       <c r="B68" s="42" t="s">
         <v>543</v>
       </c>
-      <c r="C68" s="69" t="s">
+      <c r="C68" s="71" t="s">
         <v>544</v>
       </c>
-      <c r="D68" s="69"/>
-      <c r="E68" s="70"/>
+      <c r="D68" s="71"/>
+      <c r="E68" s="72"/>
       <c r="F68" s="68"/>
       <c r="G68" s="66"/>
       <c r="H68" s="66"/>
@@ -10853,11 +10869,11 @@
       <c r="B69" s="42" t="s">
         <v>546</v>
       </c>
-      <c r="C69" s="69" t="s">
+      <c r="C69" s="71" t="s">
         <v>547</v>
       </c>
-      <c r="D69" s="69"/>
-      <c r="E69" s="70"/>
+      <c r="D69" s="71"/>
+      <c r="E69" s="72"/>
       <c r="F69" s="68"/>
       <c r="G69" s="66"/>
       <c r="H69" s="66"/>
@@ -10870,11 +10886,11 @@
       <c r="B70" s="42" t="s">
         <v>549</v>
       </c>
-      <c r="C70" s="69" t="s">
+      <c r="C70" s="71" t="s">
         <v>550</v>
       </c>
-      <c r="D70" s="69"/>
-      <c r="E70" s="70"/>
+      <c r="D70" s="71"/>
+      <c r="E70" s="72"/>
       <c r="F70" s="68"/>
       <c r="G70" s="66"/>
       <c r="H70" s="66"/>
@@ -10887,11 +10903,11 @@
       <c r="B71" s="42" t="s">
         <v>552</v>
       </c>
-      <c r="C71" s="69" t="s">
+      <c r="C71" s="71" t="s">
         <v>553</v>
       </c>
-      <c r="D71" s="69"/>
-      <c r="E71" s="70"/>
+      <c r="D71" s="71"/>
+      <c r="E71" s="72"/>
       <c r="F71" s="68"/>
       <c r="G71" s="66"/>
       <c r="H71" s="66"/>
@@ -10904,11 +10920,11 @@
       <c r="B72" s="42" t="s">
         <v>555</v>
       </c>
-      <c r="C72" s="69" t="s">
+      <c r="C72" s="71" t="s">
         <v>556</v>
       </c>
-      <c r="D72" s="69"/>
-      <c r="E72" s="70"/>
+      <c r="D72" s="71"/>
+      <c r="E72" s="72"/>
       <c r="F72" s="68"/>
       <c r="G72" s="66"/>
       <c r="H72" s="66"/>
@@ -10921,11 +10937,11 @@
       <c r="B73" s="42" t="s">
         <v>558</v>
       </c>
-      <c r="C73" s="69" t="s">
+      <c r="C73" s="71" t="s">
         <v>559</v>
       </c>
-      <c r="D73" s="69"/>
-      <c r="E73" s="70"/>
+      <c r="D73" s="71"/>
+      <c r="E73" s="72"/>
       <c r="F73" s="68"/>
       <c r="G73" s="66"/>
       <c r="H73" s="66"/>
@@ -10938,11 +10954,11 @@
       <c r="B74" s="42" t="s">
         <v>561</v>
       </c>
-      <c r="C74" s="69" t="s">
+      <c r="C74" s="71" t="s">
         <v>562</v>
       </c>
-      <c r="D74" s="69"/>
-      <c r="E74" s="70"/>
+      <c r="D74" s="71"/>
+      <c r="E74" s="72"/>
       <c r="F74" s="68"/>
       <c r="G74" s="66"/>
       <c r="H74" s="66"/>
@@ -10955,11 +10971,11 @@
       <c r="B75" s="42" t="s">
         <v>564</v>
       </c>
-      <c r="C75" s="69" t="s">
+      <c r="C75" s="71" t="s">
         <v>565</v>
       </c>
-      <c r="D75" s="69"/>
-      <c r="E75" s="70"/>
+      <c r="D75" s="71"/>
+      <c r="E75" s="72"/>
       <c r="F75" s="68"/>
       <c r="G75" s="66"/>
       <c r="H75" s="66"/>
@@ -10972,11 +10988,11 @@
       <c r="B76" s="42" t="s">
         <v>567</v>
       </c>
-      <c r="C76" s="69" t="s">
+      <c r="C76" s="71" t="s">
         <v>568</v>
       </c>
-      <c r="D76" s="69"/>
-      <c r="E76" s="70"/>
+      <c r="D76" s="71"/>
+      <c r="E76" s="72"/>
       <c r="F76" s="68"/>
       <c r="G76" s="66"/>
       <c r="H76" s="66"/>
@@ -10989,11 +11005,11 @@
       <c r="B77" s="42" t="s">
         <v>570</v>
       </c>
-      <c r="C77" s="69" t="s">
+      <c r="C77" s="71" t="s">
         <v>571</v>
       </c>
-      <c r="D77" s="69"/>
-      <c r="E77" s="70"/>
+      <c r="D77" s="71"/>
+      <c r="E77" s="72"/>
       <c r="F77" s="68"/>
       <c r="G77" s="66"/>
       <c r="H77" s="66"/>
@@ -11006,11 +11022,11 @@
       <c r="B78" s="42" t="s">
         <v>573</v>
       </c>
-      <c r="C78" s="69" t="s">
+      <c r="C78" s="71" t="s">
         <v>574</v>
       </c>
-      <c r="D78" s="69"/>
-      <c r="E78" s="70"/>
+      <c r="D78" s="71"/>
+      <c r="E78" s="72"/>
       <c r="F78" s="68"/>
       <c r="G78" s="66"/>
       <c r="H78" s="66"/>
@@ -11023,11 +11039,11 @@
       <c r="B79" s="42" t="s">
         <v>576</v>
       </c>
-      <c r="C79" s="69" t="s">
+      <c r="C79" s="71" t="s">
         <v>577</v>
       </c>
-      <c r="D79" s="69"/>
-      <c r="E79" s="70"/>
+      <c r="D79" s="71"/>
+      <c r="E79" s="72"/>
       <c r="F79" s="68"/>
       <c r="G79" s="66"/>
       <c r="H79" s="66"/>
@@ -11040,11 +11056,11 @@
       <c r="B80" s="42" t="s">
         <v>579</v>
       </c>
-      <c r="C80" s="69" t="s">
+      <c r="C80" s="71" t="s">
         <v>580</v>
       </c>
-      <c r="D80" s="69"/>
-      <c r="E80" s="70"/>
+      <c r="D80" s="71"/>
+      <c r="E80" s="72"/>
       <c r="F80" s="68"/>
       <c r="G80" s="66"/>
       <c r="H80" s="66"/>
@@ -11057,11 +11073,11 @@
       <c r="B81" s="42" t="s">
         <v>582</v>
       </c>
-      <c r="C81" s="69" t="s">
+      <c r="C81" s="71" t="s">
         <v>583</v>
       </c>
-      <c r="D81" s="69"/>
-      <c r="E81" s="70"/>
+      <c r="D81" s="71"/>
+      <c r="E81" s="72"/>
       <c r="F81" s="68"/>
       <c r="G81" s="66"/>
       <c r="H81" s="66"/>
@@ -11074,11 +11090,11 @@
       <c r="B82" t="s">
         <v>2019</v>
       </c>
-      <c r="C82" s="73" t="s">
+      <c r="C82" s="69" t="s">
         <v>2016</v>
       </c>
-      <c r="D82" s="73"/>
-      <c r="E82" s="73"/>
+      <c r="D82" s="69"/>
+      <c r="E82" s="69"/>
       <c r="F82" s="68"/>
       <c r="G82" s="66"/>
       <c r="H82" s="66"/>
@@ -11091,11 +11107,11 @@
       <c r="B83" t="s">
         <v>2020</v>
       </c>
-      <c r="C83" s="73" t="s">
+      <c r="C83" s="69" t="s">
         <v>2018</v>
       </c>
-      <c r="D83" s="73"/>
-      <c r="E83" s="73"/>
+      <c r="D83" s="69"/>
+      <c r="E83" s="69"/>
       <c r="F83" s="68"/>
       <c r="G83" s="66"/>
       <c r="H83" s="66"/>
@@ -11103,6 +11119,103 @@
     </row>
   </sheetData>
   <mergeCells count="121">
+    <mergeCell ref="F80:I80"/>
+    <mergeCell ref="F81:I81"/>
+    <mergeCell ref="F75:I75"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="F77:I77"/>
+    <mergeCell ref="F78:I78"/>
+    <mergeCell ref="F79:I79"/>
+    <mergeCell ref="F70:I70"/>
+    <mergeCell ref="F71:I71"/>
+    <mergeCell ref="F72:I72"/>
+    <mergeCell ref="F73:I73"/>
+    <mergeCell ref="F74:I74"/>
+    <mergeCell ref="F66:I66"/>
+    <mergeCell ref="F67:I67"/>
+    <mergeCell ref="F68:I68"/>
+    <mergeCell ref="F69:I69"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F65:I65"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:I33"/>
     <mergeCell ref="C82:E82"/>
     <mergeCell ref="C83:E83"/>
     <mergeCell ref="F82:I82"/>
@@ -11127,103 +11240,6 @@
     <mergeCell ref="F34:I34"/>
     <mergeCell ref="F25:I25"/>
     <mergeCell ref="C26:D26"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="C74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="C61:E61"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F65:I65"/>
-    <mergeCell ref="F66:I66"/>
-    <mergeCell ref="F67:I67"/>
-    <mergeCell ref="F68:I68"/>
-    <mergeCell ref="F69:I69"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="F63:I63"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="F80:I80"/>
-    <mergeCell ref="F81:I81"/>
-    <mergeCell ref="F75:I75"/>
-    <mergeCell ref="F76:I76"/>
-    <mergeCell ref="F77:I77"/>
-    <mergeCell ref="F78:I78"/>
-    <mergeCell ref="F79:I79"/>
-    <mergeCell ref="F70:I70"/>
-    <mergeCell ref="F71:I71"/>
-    <mergeCell ref="F72:I72"/>
-    <mergeCell ref="F73:I73"/>
-    <mergeCell ref="F74:I74"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12362,7 +12378,7 @@
       <c r="I34" s="66"/>
       <c r="J34" s="66"/>
     </row>
-    <row r="35" spans="1:10" ht="16.2" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="49" t="s">
         <v>1778</v>
       </c>
@@ -12416,19 +12432,29 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="G34:J34"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="C32:D32"/>
@@ -12441,29 +12467,19 @@
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="G31:J31"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C33:D33"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E13:F21" xr:uid="{7FAB08B6-9907-44B4-A82A-4A3E200D36A8}">
@@ -13790,23 +13806,25 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="F60:I60"/>
     <mergeCell ref="F55:I55"/>
     <mergeCell ref="F33:I33"/>
     <mergeCell ref="F35:I35"/>
@@ -13820,25 +13838,23 @@
     <mergeCell ref="F49:I49"/>
     <mergeCell ref="F50:I50"/>
     <mergeCell ref="F34:I34"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="F63:I63"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F18:I18"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="1">
@@ -18402,15 +18418,96 @@
   </sheetData>
   <dataConsolidate link="1"/>
   <mergeCells count="111">
-    <mergeCell ref="H150:K150"/>
-    <mergeCell ref="H151:K151"/>
-    <mergeCell ref="H152:K152"/>
-    <mergeCell ref="H144:K144"/>
-    <mergeCell ref="H145:K145"/>
-    <mergeCell ref="H146:K146"/>
-    <mergeCell ref="H147:K147"/>
-    <mergeCell ref="H148:K148"/>
-    <mergeCell ref="H149:K149"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H28:K28"/>
+    <mergeCell ref="H37:K37"/>
+    <mergeCell ref="H38:K38"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="H51:K51"/>
+    <mergeCell ref="H52:K52"/>
+    <mergeCell ref="H53:K53"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="H41:K41"/>
+    <mergeCell ref="H42:K42"/>
+    <mergeCell ref="H43:K43"/>
+    <mergeCell ref="H44:K44"/>
+    <mergeCell ref="H62:K62"/>
+    <mergeCell ref="H63:K63"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="H65:K65"/>
+    <mergeCell ref="H66:K66"/>
+    <mergeCell ref="H68:K68"/>
+    <mergeCell ref="H54:K54"/>
+    <mergeCell ref="H55:K55"/>
+    <mergeCell ref="H56:K56"/>
+    <mergeCell ref="H58:K58"/>
+    <mergeCell ref="H60:K60"/>
+    <mergeCell ref="H61:K61"/>
+    <mergeCell ref="H77:K77"/>
+    <mergeCell ref="H78:K78"/>
+    <mergeCell ref="H79:K79"/>
+    <mergeCell ref="H80:K80"/>
+    <mergeCell ref="H81:K81"/>
+    <mergeCell ref="H82:K82"/>
+    <mergeCell ref="H69:K69"/>
+    <mergeCell ref="H70:K70"/>
+    <mergeCell ref="H72:K72"/>
+    <mergeCell ref="H73:K73"/>
+    <mergeCell ref="H75:K75"/>
+    <mergeCell ref="H76:K76"/>
+    <mergeCell ref="H89:K89"/>
+    <mergeCell ref="H90:K90"/>
+    <mergeCell ref="H91:K91"/>
+    <mergeCell ref="H92:K92"/>
+    <mergeCell ref="H93:K93"/>
+    <mergeCell ref="H94:K94"/>
+    <mergeCell ref="H83:K83"/>
+    <mergeCell ref="H84:K84"/>
+    <mergeCell ref="H85:K85"/>
+    <mergeCell ref="H86:K86"/>
+    <mergeCell ref="H87:K87"/>
+    <mergeCell ref="H88:K88"/>
+    <mergeCell ref="H101:K101"/>
+    <mergeCell ref="H102:K102"/>
+    <mergeCell ref="H103:K103"/>
+    <mergeCell ref="H104:K104"/>
+    <mergeCell ref="H105:K105"/>
+    <mergeCell ref="H107:K107"/>
+    <mergeCell ref="H95:K95"/>
+    <mergeCell ref="H96:K96"/>
+    <mergeCell ref="H97:K97"/>
+    <mergeCell ref="H98:K98"/>
+    <mergeCell ref="H99:K99"/>
+    <mergeCell ref="H100:K100"/>
+    <mergeCell ref="H114:K114"/>
+    <mergeCell ref="H115:K115"/>
+    <mergeCell ref="H116:K116"/>
+    <mergeCell ref="H117:K117"/>
+    <mergeCell ref="H118:K118"/>
+    <mergeCell ref="H119:K119"/>
+    <mergeCell ref="H108:K108"/>
+    <mergeCell ref="H109:K109"/>
+    <mergeCell ref="H110:K110"/>
+    <mergeCell ref="H111:K111"/>
+    <mergeCell ref="H112:K112"/>
+    <mergeCell ref="H113:K113"/>
+    <mergeCell ref="H126:K126"/>
+    <mergeCell ref="H127:K127"/>
+    <mergeCell ref="H128:K128"/>
+    <mergeCell ref="H129:K129"/>
+    <mergeCell ref="H130:K130"/>
+    <mergeCell ref="H131:K131"/>
+    <mergeCell ref="H120:K120"/>
+    <mergeCell ref="H121:K121"/>
+    <mergeCell ref="H122:K122"/>
+    <mergeCell ref="H123:K123"/>
+    <mergeCell ref="H124:K124"/>
+    <mergeCell ref="H125:K125"/>
     <mergeCell ref="H138:K138"/>
     <mergeCell ref="H139:K139"/>
     <mergeCell ref="H140:K140"/>
@@ -18423,96 +18520,15 @@
     <mergeCell ref="H135:K135"/>
     <mergeCell ref="H136:K136"/>
     <mergeCell ref="H137:K137"/>
-    <mergeCell ref="H126:K126"/>
-    <mergeCell ref="H127:K127"/>
-    <mergeCell ref="H128:K128"/>
-    <mergeCell ref="H129:K129"/>
-    <mergeCell ref="H130:K130"/>
-    <mergeCell ref="H131:K131"/>
-    <mergeCell ref="H120:K120"/>
-    <mergeCell ref="H121:K121"/>
-    <mergeCell ref="H122:K122"/>
-    <mergeCell ref="H123:K123"/>
-    <mergeCell ref="H124:K124"/>
-    <mergeCell ref="H125:K125"/>
-    <mergeCell ref="H114:K114"/>
-    <mergeCell ref="H115:K115"/>
-    <mergeCell ref="H116:K116"/>
-    <mergeCell ref="H117:K117"/>
-    <mergeCell ref="H118:K118"/>
-    <mergeCell ref="H119:K119"/>
-    <mergeCell ref="H108:K108"/>
-    <mergeCell ref="H109:K109"/>
-    <mergeCell ref="H110:K110"/>
-    <mergeCell ref="H111:K111"/>
-    <mergeCell ref="H112:K112"/>
-    <mergeCell ref="H113:K113"/>
-    <mergeCell ref="H101:K101"/>
-    <mergeCell ref="H102:K102"/>
-    <mergeCell ref="H103:K103"/>
-    <mergeCell ref="H104:K104"/>
-    <mergeCell ref="H105:K105"/>
-    <mergeCell ref="H107:K107"/>
-    <mergeCell ref="H95:K95"/>
-    <mergeCell ref="H96:K96"/>
-    <mergeCell ref="H97:K97"/>
-    <mergeCell ref="H98:K98"/>
-    <mergeCell ref="H99:K99"/>
-    <mergeCell ref="H100:K100"/>
-    <mergeCell ref="H89:K89"/>
-    <mergeCell ref="H90:K90"/>
-    <mergeCell ref="H91:K91"/>
-    <mergeCell ref="H92:K92"/>
-    <mergeCell ref="H93:K93"/>
-    <mergeCell ref="H94:K94"/>
-    <mergeCell ref="H83:K83"/>
-    <mergeCell ref="H84:K84"/>
-    <mergeCell ref="H85:K85"/>
-    <mergeCell ref="H86:K86"/>
-    <mergeCell ref="H87:K87"/>
-    <mergeCell ref="H88:K88"/>
-    <mergeCell ref="H77:K77"/>
-    <mergeCell ref="H78:K78"/>
-    <mergeCell ref="H79:K79"/>
-    <mergeCell ref="H80:K80"/>
-    <mergeCell ref="H81:K81"/>
-    <mergeCell ref="H82:K82"/>
-    <mergeCell ref="H69:K69"/>
-    <mergeCell ref="H70:K70"/>
-    <mergeCell ref="H72:K72"/>
-    <mergeCell ref="H73:K73"/>
-    <mergeCell ref="H75:K75"/>
-    <mergeCell ref="H76:K76"/>
-    <mergeCell ref="H62:K62"/>
-    <mergeCell ref="H63:K63"/>
-    <mergeCell ref="H64:K64"/>
-    <mergeCell ref="H65:K65"/>
-    <mergeCell ref="H66:K66"/>
-    <mergeCell ref="H68:K68"/>
-    <mergeCell ref="H54:K54"/>
-    <mergeCell ref="H55:K55"/>
-    <mergeCell ref="H56:K56"/>
-    <mergeCell ref="H58:K58"/>
-    <mergeCell ref="H60:K60"/>
-    <mergeCell ref="H61:K61"/>
-    <mergeCell ref="H51:K51"/>
-    <mergeCell ref="H52:K52"/>
-    <mergeCell ref="H53:K53"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="H41:K41"/>
-    <mergeCell ref="H42:K42"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="H44:K44"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="H28:K28"/>
-    <mergeCell ref="H37:K37"/>
-    <mergeCell ref="H38:K38"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="H150:K150"/>
+    <mergeCell ref="H151:K151"/>
+    <mergeCell ref="H152:K152"/>
+    <mergeCell ref="H144:K144"/>
+    <mergeCell ref="H145:K145"/>
+    <mergeCell ref="H146:K146"/>
+    <mergeCell ref="H147:K147"/>
+    <mergeCell ref="H148:K148"/>
+    <mergeCell ref="H149:K149"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -21091,6 +21107,21 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="F113:I113"/>
+    <mergeCell ref="C118:D118"/>
+    <mergeCell ref="C113:D113"/>
+    <mergeCell ref="C114:D114"/>
+    <mergeCell ref="C115:D115"/>
+    <mergeCell ref="C116:D116"/>
+    <mergeCell ref="C117:D117"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="C119:D119"/>
+    <mergeCell ref="C120:D120"/>
+    <mergeCell ref="C121:D121"/>
+    <mergeCell ref="C122:D122"/>
+    <mergeCell ref="C123:D123"/>
+    <mergeCell ref="C124:D124"/>
+    <mergeCell ref="C125:D125"/>
     <mergeCell ref="F109:I109"/>
     <mergeCell ref="F110:I110"/>
     <mergeCell ref="F111:I111"/>
@@ -21099,21 +21130,6 @@
     <mergeCell ref="C110:D110"/>
     <mergeCell ref="C111:D111"/>
     <mergeCell ref="C112:D112"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="C119:D119"/>
-    <mergeCell ref="C120:D120"/>
-    <mergeCell ref="C121:D121"/>
-    <mergeCell ref="C122:D122"/>
-    <mergeCell ref="C123:D123"/>
-    <mergeCell ref="C124:D124"/>
-    <mergeCell ref="C125:D125"/>
-    <mergeCell ref="F113:I113"/>
-    <mergeCell ref="C118:D118"/>
-    <mergeCell ref="C113:D113"/>
-    <mergeCell ref="C114:D114"/>
-    <mergeCell ref="C115:D115"/>
-    <mergeCell ref="C116:D116"/>
-    <mergeCell ref="C117:D117"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -21929,6 +21945,15 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="H54:K54"/>
+    <mergeCell ref="H55:K55"/>
+    <mergeCell ref="H56:K56"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="H51:K51"/>
+    <mergeCell ref="H52:K52"/>
+    <mergeCell ref="H53:K53"/>
     <mergeCell ref="H44:K44"/>
     <mergeCell ref="H13:K13"/>
     <mergeCell ref="H14:K14"/>
@@ -21941,15 +21966,6 @@
     <mergeCell ref="H41:K41"/>
     <mergeCell ref="H42:K42"/>
     <mergeCell ref="H43:K43"/>
-    <mergeCell ref="H54:K54"/>
-    <mergeCell ref="H55:K55"/>
-    <mergeCell ref="H56:K56"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="H48:K48"/>
-    <mergeCell ref="H51:K51"/>
-    <mergeCell ref="H52:K52"/>
-    <mergeCell ref="H53:K53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22298,14 +22314,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="H22:K22"/>
     <mergeCell ref="H33:K33"/>
     <mergeCell ref="H34:K34"/>
     <mergeCell ref="H35:K35"/>
@@ -22315,6 +22323,14 @@
     <mergeCell ref="H30:K30"/>
     <mergeCell ref="H31:K31"/>
     <mergeCell ref="H32:K32"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="H22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -22664,6 +22680,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="H31:K31"/>
+    <mergeCell ref="H32:K32"/>
+    <mergeCell ref="H33:K33"/>
+    <mergeCell ref="H34:K34"/>
+    <mergeCell ref="H35:K35"/>
     <mergeCell ref="H30:K30"/>
     <mergeCell ref="H16:K16"/>
     <mergeCell ref="H17:K17"/>
@@ -22676,11 +22697,6 @@
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="H25:K25"/>
     <mergeCell ref="H27:K27"/>
-    <mergeCell ref="H31:K31"/>
-    <mergeCell ref="H32:K32"/>
-    <mergeCell ref="H33:K33"/>
-    <mergeCell ref="H34:K34"/>
-    <mergeCell ref="H35:K35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -23741,10 +23757,10 @@
       <c r="B44" s="48" t="s">
         <v>1163</v>
       </c>
-      <c r="C44" s="73" t="s">
+      <c r="C44" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D44" s="73"/>
+      <c r="D44" s="69"/>
       <c r="E44" s="5" t="s">
         <v>1164</v>
       </c>
@@ -23758,10 +23774,10 @@
       <c r="B45" s="48" t="s">
         <v>1165</v>
       </c>
-      <c r="C45" s="73" t="s">
+      <c r="C45" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D45" s="73"/>
+      <c r="D45" s="69"/>
       <c r="E45" s="5" t="s">
         <v>1166</v>
       </c>
@@ -23775,10 +23791,10 @@
       <c r="B46" s="48" t="s">
         <v>1167</v>
       </c>
-      <c r="C46" s="73" t="s">
+      <c r="C46" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D46" s="73"/>
+      <c r="D46" s="69"/>
       <c r="E46" s="5" t="s">
         <v>1168</v>
       </c>
@@ -23792,10 +23808,10 @@
       <c r="B47" s="48" t="s">
         <v>1169</v>
       </c>
-      <c r="C47" s="73" t="s">
+      <c r="C47" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D47" s="73"/>
+      <c r="D47" s="69"/>
       <c r="E47" s="5" t="s">
         <v>1170</v>
       </c>
@@ -23809,10 +23825,10 @@
       <c r="B48" s="48" t="s">
         <v>1171</v>
       </c>
-      <c r="C48" s="73" t="s">
+      <c r="C48" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D48" s="73"/>
+      <c r="D48" s="69"/>
       <c r="E48" s="5" t="s">
         <v>1172</v>
       </c>
@@ -23826,10 +23842,10 @@
       <c r="B49" s="48" t="s">
         <v>1173</v>
       </c>
-      <c r="C49" s="73" t="s">
+      <c r="C49" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D49" s="73"/>
+      <c r="D49" s="69"/>
       <c r="E49" s="5" t="s">
         <v>1174</v>
       </c>
@@ -23843,10 +23859,10 @@
       <c r="B50" s="48" t="s">
         <v>1175</v>
       </c>
-      <c r="C50" s="73" t="s">
+      <c r="C50" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D50" s="73"/>
+      <c r="D50" s="69"/>
       <c r="E50" s="5" t="s">
         <v>1176</v>
       </c>
@@ -23860,10 +23876,10 @@
       <c r="B51" s="48" t="s">
         <v>1177</v>
       </c>
-      <c r="C51" s="73" t="s">
+      <c r="C51" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D51" s="73"/>
+      <c r="D51" s="69"/>
       <c r="E51" s="5" t="s">
         <v>1178</v>
       </c>
@@ -23877,10 +23893,10 @@
       <c r="B52" s="48" t="s">
         <v>1179</v>
       </c>
-      <c r="C52" s="73" t="s">
+      <c r="C52" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D52" s="73"/>
+      <c r="D52" s="69"/>
       <c r="E52" s="5" t="s">
         <v>1180</v>
       </c>
@@ -23894,10 +23910,10 @@
       <c r="B53" s="48" t="s">
         <v>1181</v>
       </c>
-      <c r="C53" s="73" t="s">
+      <c r="C53" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D53" s="73"/>
+      <c r="D53" s="69"/>
       <c r="E53" s="5" t="s">
         <v>1182</v>
       </c>
@@ -23911,10 +23927,10 @@
       <c r="B54" s="48" t="s">
         <v>1183</v>
       </c>
-      <c r="C54" s="73" t="s">
+      <c r="C54" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D54" s="73"/>
+      <c r="D54" s="69"/>
       <c r="E54" s="5" t="s">
         <v>1184</v>
       </c>
@@ -23928,10 +23944,10 @@
       <c r="B55" s="48" t="s">
         <v>1185</v>
       </c>
-      <c r="C55" s="73" t="s">
+      <c r="C55" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D55" s="73"/>
+      <c r="D55" s="69"/>
       <c r="E55" s="5" t="s">
         <v>1186</v>
       </c>
@@ -23945,10 +23961,10 @@
       <c r="B56" s="48" t="s">
         <v>1187</v>
       </c>
-      <c r="C56" s="73" t="s">
+      <c r="C56" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D56" s="73"/>
+      <c r="D56" s="69"/>
       <c r="E56" s="5" t="s">
         <v>1188</v>
       </c>
@@ -23962,10 +23978,10 @@
       <c r="B57" s="48" t="s">
         <v>1189</v>
       </c>
-      <c r="C57" s="73" t="s">
+      <c r="C57" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D57" s="73"/>
+      <c r="D57" s="69"/>
       <c r="E57" s="5" t="s">
         <v>1190</v>
       </c>
@@ -23979,10 +23995,10 @@
       <c r="B58" s="48" t="s">
         <v>1191</v>
       </c>
-      <c r="C58" s="73" t="s">
+      <c r="C58" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D58" s="73"/>
+      <c r="D58" s="69"/>
       <c r="E58" s="5" t="s">
         <v>1192</v>
       </c>
@@ -23996,10 +24012,10 @@
       <c r="B59" s="48" t="s">
         <v>1193</v>
       </c>
-      <c r="C59" s="73" t="s">
+      <c r="C59" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D59" s="73"/>
+      <c r="D59" s="69"/>
       <c r="E59" s="5" t="s">
         <v>1194</v>
       </c>
@@ -24013,10 +24029,10 @@
       <c r="B60" s="48" t="s">
         <v>1195</v>
       </c>
-      <c r="C60" s="73" t="s">
+      <c r="C60" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D60" s="73"/>
+      <c r="D60" s="69"/>
       <c r="E60" s="5" t="s">
         <v>1196</v>
       </c>
@@ -24030,10 +24046,10 @@
       <c r="B61" s="48" t="s">
         <v>1197</v>
       </c>
-      <c r="C61" s="73" t="s">
+      <c r="C61" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D61" s="73"/>
+      <c r="D61" s="69"/>
       <c r="E61" s="5" t="s">
         <v>1198</v>
       </c>
@@ -24047,10 +24063,10 @@
       <c r="B62" s="48" t="s">
         <v>1199</v>
       </c>
-      <c r="C62" s="73" t="s">
+      <c r="C62" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D62" s="73"/>
+      <c r="D62" s="69"/>
       <c r="E62" s="5" t="s">
         <v>1200</v>
       </c>
@@ -24064,10 +24080,10 @@
       <c r="B63" s="48" t="s">
         <v>1201</v>
       </c>
-      <c r="C63" s="73" t="s">
+      <c r="C63" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D63" s="73"/>
+      <c r="D63" s="69"/>
       <c r="E63" s="5" t="s">
         <v>1202</v>
       </c>
@@ -24081,10 +24097,10 @@
       <c r="B64" s="48" t="s">
         <v>1203</v>
       </c>
-      <c r="C64" s="73" t="s">
+      <c r="C64" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D64" s="73"/>
+      <c r="D64" s="69"/>
       <c r="E64" s="5" t="s">
         <v>1204</v>
       </c>
@@ -24098,10 +24114,10 @@
       <c r="B65" s="48" t="s">
         <v>1205</v>
       </c>
-      <c r="C65" s="73" t="s">
+      <c r="C65" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D65" s="73"/>
+      <c r="D65" s="69"/>
       <c r="E65" s="5" t="s">
         <v>1206</v>
       </c>
@@ -24115,10 +24131,10 @@
       <c r="B66" s="48" t="s">
         <v>1207</v>
       </c>
-      <c r="C66" s="73" t="s">
+      <c r="C66" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D66" s="73"/>
+      <c r="D66" s="69"/>
       <c r="E66" s="5" t="s">
         <v>1208</v>
       </c>
@@ -24132,10 +24148,10 @@
       <c r="B67" s="48" t="s">
         <v>1209</v>
       </c>
-      <c r="C67" s="73" t="s">
+      <c r="C67" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D67" s="73"/>
+      <c r="D67" s="69"/>
       <c r="E67" s="5" t="s">
         <v>1210</v>
       </c>
@@ -24149,10 +24165,10 @@
       <c r="B68" s="48" t="s">
         <v>1211</v>
       </c>
-      <c r="C68" s="73" t="s">
+      <c r="C68" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D68" s="73"/>
+      <c r="D68" s="69"/>
       <c r="E68" s="5" t="s">
         <v>1212</v>
       </c>
@@ -24166,10 +24182,10 @@
       <c r="B69" s="48" t="s">
         <v>1213</v>
       </c>
-      <c r="C69" s="73" t="s">
+      <c r="C69" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D69" s="73"/>
+      <c r="D69" s="69"/>
       <c r="E69" s="5" t="s">
         <v>1214</v>
       </c>
@@ -24183,10 +24199,10 @@
       <c r="B70" s="48" t="s">
         <v>1215</v>
       </c>
-      <c r="C70" s="73" t="s">
+      <c r="C70" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D70" s="73"/>
+      <c r="D70" s="69"/>
       <c r="E70" s="5" t="s">
         <v>1216</v>
       </c>
@@ -24200,10 +24216,10 @@
       <c r="B71" s="48" t="s">
         <v>1217</v>
       </c>
-      <c r="C71" s="73" t="s">
+      <c r="C71" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D71" s="73"/>
+      <c r="D71" s="69"/>
       <c r="E71" s="5" t="s">
         <v>1218</v>
       </c>
@@ -24217,10 +24233,10 @@
       <c r="B72" s="48" t="s">
         <v>1219</v>
       </c>
-      <c r="C72" s="73" t="s">
+      <c r="C72" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D72" s="73"/>
+      <c r="D72" s="69"/>
       <c r="E72" s="5" t="s">
         <v>1220</v>
       </c>
@@ -24234,10 +24250,10 @@
       <c r="B73" s="48" t="s">
         <v>1221</v>
       </c>
-      <c r="C73" s="73" t="s">
+      <c r="C73" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D73" s="73"/>
+      <c r="D73" s="69"/>
       <c r="E73" s="5" t="s">
         <v>1222</v>
       </c>
@@ -24251,10 +24267,10 @@
       <c r="B74" s="48" t="s">
         <v>1223</v>
       </c>
-      <c r="C74" s="73" t="s">
+      <c r="C74" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D74" s="73"/>
+      <c r="D74" s="69"/>
       <c r="E74" s="5" t="s">
         <v>1224</v>
       </c>
@@ -24268,10 +24284,10 @@
       <c r="B75" s="48" t="s">
         <v>1225</v>
       </c>
-      <c r="C75" s="73" t="s">
+      <c r="C75" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D75" s="73"/>
+      <c r="D75" s="69"/>
       <c r="E75" s="5" t="s">
         <v>1226</v>
       </c>
@@ -24285,10 +24301,10 @@
       <c r="B76" s="48" t="s">
         <v>1227</v>
       </c>
-      <c r="C76" s="73" t="s">
+      <c r="C76" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D76" s="73"/>
+      <c r="D76" s="69"/>
       <c r="E76" s="5" t="s">
         <v>1228</v>
       </c>
@@ -24302,10 +24318,10 @@
       <c r="B77" s="48" t="s">
         <v>1229</v>
       </c>
-      <c r="C77" s="73" t="s">
+      <c r="C77" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D77" s="73"/>
+      <c r="D77" s="69"/>
       <c r="E77" s="5" t="s">
         <v>1230</v>
       </c>
@@ -24319,10 +24335,10 @@
       <c r="B78" s="48" t="s">
         <v>1231</v>
       </c>
-      <c r="C78" s="73" t="s">
+      <c r="C78" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D78" s="73"/>
+      <c r="D78" s="69"/>
       <c r="E78" s="5" t="s">
         <v>1232</v>
       </c>
@@ -24336,10 +24352,10 @@
       <c r="B79" s="48" t="s">
         <v>1233</v>
       </c>
-      <c r="C79" s="73" t="s">
+      <c r="C79" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D79" s="73"/>
+      <c r="D79" s="69"/>
       <c r="E79" s="5" t="s">
         <v>1234</v>
       </c>
@@ -24353,10 +24369,10 @@
       <c r="B80" s="48" t="s">
         <v>1235</v>
       </c>
-      <c r="C80" s="73" t="s">
+      <c r="C80" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D80" s="73"/>
+      <c r="D80" s="69"/>
       <c r="E80" s="5" t="s">
         <v>1236</v>
       </c>
@@ -24370,10 +24386,10 @@
       <c r="B81" s="48" t="s">
         <v>1237</v>
       </c>
-      <c r="C81" s="73" t="s">
+      <c r="C81" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D81" s="73"/>
+      <c r="D81" s="69"/>
       <c r="E81" s="5" t="s">
         <v>1238</v>
       </c>
@@ -24387,10 +24403,10 @@
       <c r="B82" s="48" t="s">
         <v>1239</v>
       </c>
-      <c r="C82" s="73" t="s">
+      <c r="C82" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D82" s="73"/>
+      <c r="D82" s="69"/>
       <c r="E82" s="5" t="s">
         <v>1240</v>
       </c>
@@ -24404,10 +24420,10 @@
       <c r="B83" s="48" t="s">
         <v>1268</v>
       </c>
-      <c r="C83" s="73" t="s">
+      <c r="C83" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D83" s="73"/>
+      <c r="D83" s="69"/>
       <c r="E83" s="5" t="s">
         <v>1234</v>
       </c>
@@ -24421,10 +24437,10 @@
       <c r="B84" s="48" t="s">
         <v>1269</v>
       </c>
-      <c r="C84" s="73" t="s">
+      <c r="C84" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D84" s="73"/>
+      <c r="D84" s="69"/>
       <c r="E84" s="5" t="s">
         <v>1236</v>
       </c>
@@ -24438,10 +24454,10 @@
       <c r="B85" s="48" t="s">
         <v>1270</v>
       </c>
-      <c r="C85" s="73" t="s">
+      <c r="C85" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D85" s="73"/>
+      <c r="D85" s="69"/>
       <c r="E85" s="5" t="s">
         <v>1238</v>
       </c>
@@ -24455,10 +24471,10 @@
       <c r="B86" s="48" t="s">
         <v>1271</v>
       </c>
-      <c r="C86" s="73" t="s">
+      <c r="C86" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D86" s="73"/>
+      <c r="D86" s="69"/>
       <c r="E86" s="5" t="s">
         <v>1241</v>
       </c>
@@ -24472,10 +24488,10 @@
       <c r="B87" s="48" t="s">
         <v>1242</v>
       </c>
-      <c r="C87" s="73" t="s">
+      <c r="C87" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D87" s="73"/>
+      <c r="D87" s="69"/>
       <c r="E87" s="5" t="s">
         <v>1234</v>
       </c>
@@ -24489,10 +24505,10 @@
       <c r="B88" s="48" t="s">
         <v>1243</v>
       </c>
-      <c r="C88" s="73" t="s">
+      <c r="C88" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D88" s="73"/>
+      <c r="D88" s="69"/>
       <c r="E88" s="5" t="s">
         <v>1236</v>
       </c>
@@ -24506,10 +24522,10 @@
       <c r="B89" s="48" t="s">
         <v>1244</v>
       </c>
-      <c r="C89" s="73" t="s">
+      <c r="C89" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D89" s="73"/>
+      <c r="D89" s="69"/>
       <c r="E89" s="5" t="s">
         <v>1238</v>
       </c>
@@ -24523,10 +24539,10 @@
       <c r="B90" s="48" t="s">
         <v>1245</v>
       </c>
-      <c r="C90" s="73" t="s">
+      <c r="C90" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D90" s="73"/>
+      <c r="D90" s="69"/>
       <c r="E90" s="5" t="s">
         <v>1241</v>
       </c>
@@ -24540,10 +24556,10 @@
       <c r="B91" s="48" t="s">
         <v>1272</v>
       </c>
-      <c r="C91" s="73" t="s">
+      <c r="C91" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D91" s="73"/>
+      <c r="D91" s="69"/>
       <c r="E91" s="5" t="s">
         <v>1234</v>
       </c>
@@ -24557,10 +24573,10 @@
       <c r="B92" s="48" t="s">
         <v>1273</v>
       </c>
-      <c r="C92" s="73" t="s">
+      <c r="C92" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D92" s="73"/>
+      <c r="D92" s="69"/>
       <c r="E92" s="5" t="s">
         <v>1236</v>
       </c>
@@ -24574,10 +24590,10 @@
       <c r="B93" s="48" t="s">
         <v>1274</v>
       </c>
-      <c r="C93" s="73" t="s">
+      <c r="C93" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D93" s="73"/>
+      <c r="D93" s="69"/>
       <c r="E93" s="5" t="s">
         <v>1238</v>
       </c>
@@ -24591,10 +24607,10 @@
       <c r="B94" s="48" t="s">
         <v>1275</v>
       </c>
-      <c r="C94" s="73" t="s">
+      <c r="C94" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D94" s="73"/>
+      <c r="D94" s="69"/>
       <c r="E94" s="5" t="s">
         <v>1241</v>
       </c>
@@ -24608,10 +24624,10 @@
       <c r="B95" s="48" t="s">
         <v>1276</v>
       </c>
-      <c r="C95" s="73" t="s">
+      <c r="C95" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D95" s="73"/>
+      <c r="D95" s="69"/>
       <c r="E95" s="5" t="s">
         <v>1246</v>
       </c>
@@ -24625,10 +24641,10 @@
       <c r="B96" s="48" t="s">
         <v>1247</v>
       </c>
-      <c r="C96" s="73" t="s">
+      <c r="C96" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D96" s="73"/>
+      <c r="D96" s="69"/>
       <c r="E96" s="5" t="s">
         <v>1248</v>
       </c>
@@ -24642,10 +24658,10 @@
       <c r="B97" s="48" t="s">
         <v>1249</v>
       </c>
-      <c r="C97" s="73" t="s">
+      <c r="C97" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D97" s="73"/>
+      <c r="D97" s="69"/>
       <c r="E97" s="5" t="s">
         <v>1250</v>
       </c>
@@ -24659,10 +24675,10 @@
       <c r="B98" s="48" t="s">
         <v>1251</v>
       </c>
-      <c r="C98" s="73" t="s">
+      <c r="C98" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D98" s="73"/>
+      <c r="D98" s="69"/>
       <c r="E98" s="5" t="s">
         <v>1252</v>
       </c>
@@ -24676,10 +24692,10 @@
       <c r="B99" s="48" t="s">
         <v>1253</v>
       </c>
-      <c r="C99" s="73" t="s">
+      <c r="C99" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D99" s="73"/>
+      <c r="D99" s="69"/>
       <c r="E99" s="5" t="s">
         <v>1254</v>
       </c>
@@ -24693,10 +24709,10 @@
       <c r="B100" s="48" t="s">
         <v>1255</v>
       </c>
-      <c r="C100" s="73" t="s">
+      <c r="C100" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D100" s="73"/>
+      <c r="D100" s="69"/>
       <c r="E100" s="5" t="s">
         <v>1256</v>
       </c>
@@ -24710,10 +24726,10 @@
       <c r="B101" s="48" t="s">
         <v>1257</v>
       </c>
-      <c r="C101" s="73" t="s">
+      <c r="C101" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D101" s="73"/>
+      <c r="D101" s="69"/>
       <c r="E101" s="5" t="s">
         <v>1258</v>
       </c>
@@ -24727,10 +24743,10 @@
       <c r="B102" s="48" t="s">
         <v>1259</v>
       </c>
-      <c r="C102" s="73" t="s">
+      <c r="C102" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D102" s="73"/>
+      <c r="D102" s="69"/>
       <c r="E102" s="5" t="s">
         <v>1252</v>
       </c>
@@ -24744,10 +24760,10 @@
       <c r="B103" s="48" t="s">
         <v>1260</v>
       </c>
-      <c r="C103" s="73" t="s">
+      <c r="C103" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D103" s="73"/>
+      <c r="D103" s="69"/>
       <c r="E103" s="5" t="s">
         <v>1254</v>
       </c>
@@ -24761,10 +24777,10 @@
       <c r="B104" s="48" t="s">
         <v>1261</v>
       </c>
-      <c r="C104" s="73" t="s">
+      <c r="C104" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D104" s="73"/>
+      <c r="D104" s="69"/>
       <c r="E104" s="5" t="s">
         <v>1256</v>
       </c>
@@ -24778,10 +24794,10 @@
       <c r="B105" s="48" t="s">
         <v>1262</v>
       </c>
-      <c r="C105" s="73" t="s">
+      <c r="C105" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D105" s="73"/>
+      <c r="D105" s="69"/>
       <c r="E105" s="5" t="s">
         <v>1258</v>
       </c>
@@ -24795,10 +24811,10 @@
       <c r="B106" s="48" t="s">
         <v>1263</v>
       </c>
-      <c r="C106" s="73" t="s">
+      <c r="C106" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D106" s="73"/>
+      <c r="D106" s="69"/>
       <c r="E106" s="5" t="s">
         <v>1264</v>
       </c>
@@ -24812,10 +24828,10 @@
       <c r="B107" s="48" t="s">
         <v>1265</v>
       </c>
-      <c r="C107" s="73" t="s">
+      <c r="C107" s="69" t="s">
         <v>1277</v>
       </c>
-      <c r="D107" s="73"/>
+      <c r="D107" s="69"/>
       <c r="E107" s="5" t="s">
         <v>1266</v>
       </c>
@@ -24826,48 +24842,109 @@
     </row>
   </sheetData>
   <mergeCells count="169">
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="F38:I38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F104:I104"/>
+    <mergeCell ref="F105:I105"/>
+    <mergeCell ref="F106:I106"/>
+    <mergeCell ref="F107:I107"/>
+    <mergeCell ref="F99:I99"/>
+    <mergeCell ref="F100:I100"/>
+    <mergeCell ref="F101:I101"/>
+    <mergeCell ref="F102:I102"/>
+    <mergeCell ref="F103:I103"/>
+    <mergeCell ref="F94:I94"/>
+    <mergeCell ref="F95:I95"/>
+    <mergeCell ref="F96:I96"/>
+    <mergeCell ref="F97:I97"/>
+    <mergeCell ref="F98:I98"/>
+    <mergeCell ref="F89:I89"/>
+    <mergeCell ref="F90:I90"/>
+    <mergeCell ref="F91:I91"/>
+    <mergeCell ref="F92:I92"/>
+    <mergeCell ref="F93:I93"/>
+    <mergeCell ref="F84:I84"/>
+    <mergeCell ref="F85:I85"/>
+    <mergeCell ref="F86:I86"/>
+    <mergeCell ref="F87:I87"/>
+    <mergeCell ref="F88:I88"/>
+    <mergeCell ref="F79:I79"/>
+    <mergeCell ref="F80:I80"/>
+    <mergeCell ref="F81:I81"/>
+    <mergeCell ref="F82:I82"/>
+    <mergeCell ref="F83:I83"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="F65:I65"/>
+    <mergeCell ref="F66:I66"/>
+    <mergeCell ref="F67:I67"/>
+    <mergeCell ref="F68:I68"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="C78:D78"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F74:I74"/>
+    <mergeCell ref="F75:I75"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="F77:I77"/>
+    <mergeCell ref="F78:I78"/>
+    <mergeCell ref="F69:I69"/>
+    <mergeCell ref="F70:I70"/>
+    <mergeCell ref="F71:I71"/>
+    <mergeCell ref="F72:I72"/>
+    <mergeCell ref="F73:I73"/>
+    <mergeCell ref="C73:D73"/>
+    <mergeCell ref="C74:D74"/>
+    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C88:D88"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="C90:D90"/>
+    <mergeCell ref="C91:D91"/>
+    <mergeCell ref="C92:D92"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="C86:D86"/>
+    <mergeCell ref="C87:D87"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="C98:D98"/>
+    <mergeCell ref="C99:D99"/>
+    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="C101:D101"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C93:D93"/>
+    <mergeCell ref="C94:D94"/>
+    <mergeCell ref="C95:D95"/>
+    <mergeCell ref="C96:D96"/>
+    <mergeCell ref="C97:D97"/>
+    <mergeCell ref="C103:D103"/>
+    <mergeCell ref="C104:D104"/>
+    <mergeCell ref="C105:D105"/>
+    <mergeCell ref="C106:D106"/>
+    <mergeCell ref="C77:D77"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="C71:D71"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="C67:D67"/>
     <mergeCell ref="C58:D58"/>
     <mergeCell ref="C59:D59"/>
     <mergeCell ref="C60:D60"/>
@@ -24892,109 +24969,48 @@
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="F44:I44"/>
-    <mergeCell ref="C77:D77"/>
-    <mergeCell ref="C68:D68"/>
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="C71:D71"/>
-    <mergeCell ref="C72:D72"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="C107:D107"/>
-    <mergeCell ref="C98:D98"/>
-    <mergeCell ref="C99:D99"/>
-    <mergeCell ref="C100:D100"/>
-    <mergeCell ref="C101:D101"/>
-    <mergeCell ref="C102:D102"/>
-    <mergeCell ref="C93:D93"/>
-    <mergeCell ref="C94:D94"/>
-    <mergeCell ref="C95:D95"/>
-    <mergeCell ref="C96:D96"/>
-    <mergeCell ref="C97:D97"/>
-    <mergeCell ref="C103:D103"/>
-    <mergeCell ref="C104:D104"/>
-    <mergeCell ref="C105:D105"/>
-    <mergeCell ref="C106:D106"/>
-    <mergeCell ref="C88:D88"/>
-    <mergeCell ref="C89:D89"/>
-    <mergeCell ref="C90:D90"/>
-    <mergeCell ref="C91:D91"/>
-    <mergeCell ref="C92:D92"/>
-    <mergeCell ref="C83:D83"/>
-    <mergeCell ref="C84:D84"/>
-    <mergeCell ref="C85:D85"/>
-    <mergeCell ref="C86:D86"/>
-    <mergeCell ref="C87:D87"/>
-    <mergeCell ref="C78:D78"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C82:D82"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F74:I74"/>
-    <mergeCell ref="F75:I75"/>
-    <mergeCell ref="F76:I76"/>
-    <mergeCell ref="F77:I77"/>
-    <mergeCell ref="F78:I78"/>
-    <mergeCell ref="F69:I69"/>
-    <mergeCell ref="F70:I70"/>
-    <mergeCell ref="F71:I71"/>
-    <mergeCell ref="F72:I72"/>
-    <mergeCell ref="F73:I73"/>
-    <mergeCell ref="C73:D73"/>
-    <mergeCell ref="C74:D74"/>
-    <mergeCell ref="C75:D75"/>
-    <mergeCell ref="C76:D76"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="F65:I65"/>
-    <mergeCell ref="F66:I66"/>
-    <mergeCell ref="F67:I67"/>
-    <mergeCell ref="F68:I68"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="F63:I63"/>
-    <mergeCell ref="F84:I84"/>
-    <mergeCell ref="F85:I85"/>
-    <mergeCell ref="F86:I86"/>
-    <mergeCell ref="F87:I87"/>
-    <mergeCell ref="F88:I88"/>
-    <mergeCell ref="F79:I79"/>
-    <mergeCell ref="F80:I80"/>
-    <mergeCell ref="F81:I81"/>
-    <mergeCell ref="F82:I82"/>
-    <mergeCell ref="F83:I83"/>
-    <mergeCell ref="F94:I94"/>
-    <mergeCell ref="F95:I95"/>
-    <mergeCell ref="F96:I96"/>
-    <mergeCell ref="F97:I97"/>
-    <mergeCell ref="F98:I98"/>
-    <mergeCell ref="F89:I89"/>
-    <mergeCell ref="F90:I90"/>
-    <mergeCell ref="F91:I91"/>
-    <mergeCell ref="F92:I92"/>
-    <mergeCell ref="F93:I93"/>
-    <mergeCell ref="F104:I104"/>
-    <mergeCell ref="F105:I105"/>
-    <mergeCell ref="F106:I106"/>
-    <mergeCell ref="F107:I107"/>
-    <mergeCell ref="F99:I99"/>
-    <mergeCell ref="F100:I100"/>
-    <mergeCell ref="F101:I101"/>
-    <mergeCell ref="F102:I102"/>
-    <mergeCell ref="F103:I103"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F29:I29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -25949,6 +25965,18 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D22:G22"/>
     <mergeCell ref="D30:G30"/>
     <mergeCell ref="D24:G24"/>
     <mergeCell ref="D25:G25"/>
@@ -25956,18 +25984,6 @@
     <mergeCell ref="D27:G27"/>
     <mergeCell ref="D28:G28"/>
     <mergeCell ref="D29:G29"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="D17:G17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -27122,210 +27138,210 @@
         <v>1036</v>
       </c>
       <c r="D14" s="67"/>
-      <c r="E14" s="71"/>
-      <c r="F14" s="72" t="s">
+      <c r="E14" s="70"/>
+      <c r="F14" s="73" t="s">
         <v>463</v>
       </c>
-      <c r="G14" s="72"/>
-      <c r="H14" s="72"/>
-      <c r="I14" s="72"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="73"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="75" t="s">
+      <c r="A15" s="74" t="s">
         <v>1037</v>
       </c>
       <c r="B15" s="42" t="s">
         <v>1038</v>
       </c>
-      <c r="C15" s="69" t="s">
+      <c r="C15" s="71" t="s">
         <v>1039</v>
       </c>
-      <c r="D15" s="69"/>
-      <c r="E15" s="70"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="72"/>
       <c r="F15" s="68"/>
       <c r="G15" s="66"/>
       <c r="H15" s="66"/>
       <c r="I15" s="66"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="75"/>
+      <c r="A16" s="74"/>
       <c r="B16" s="42" t="s">
         <v>1040</v>
       </c>
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="71" t="s">
         <v>1041</v>
       </c>
-      <c r="D16" s="69"/>
-      <c r="E16" s="70"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="72"/>
       <c r="F16" s="68"/>
       <c r="G16" s="66"/>
       <c r="H16" s="66"/>
       <c r="I16" s="66"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="75"/>
+      <c r="A17" s="74"/>
       <c r="B17" s="42" t="s">
         <v>1042</v>
       </c>
-      <c r="C17" s="69" t="s">
+      <c r="C17" s="71" t="s">
         <v>1043</v>
       </c>
-      <c r="D17" s="69"/>
-      <c r="E17" s="70"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="72"/>
       <c r="F17" s="68"/>
       <c r="G17" s="66"/>
       <c r="H17" s="66"/>
       <c r="I17" s="66"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="75"/>
+      <c r="A18" s="74"/>
       <c r="B18" s="42" t="s">
         <v>1044</v>
       </c>
-      <c r="C18" s="70" t="s">
+      <c r="C18" s="72" t="s">
         <v>1045</v>
       </c>
-      <c r="D18" s="70"/>
-      <c r="E18" s="70"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="72"/>
       <c r="F18" s="68"/>
       <c r="G18" s="66"/>
       <c r="H18" s="66"/>
       <c r="I18" s="66"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="75"/>
+      <c r="A19" s="74"/>
       <c r="B19" s="42" t="s">
         <v>1046</v>
       </c>
-      <c r="C19" s="70" t="s">
+      <c r="C19" s="72" t="s">
         <v>1047</v>
       </c>
-      <c r="D19" s="70"/>
-      <c r="E19" s="70"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
       <c r="F19" s="68"/>
       <c r="G19" s="66"/>
       <c r="H19" s="66"/>
       <c r="I19" s="66"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="76" t="s">
+      <c r="A20" s="75" t="s">
         <v>1048</v>
       </c>
       <c r="B20" s="42" t="s">
         <v>1049</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="72" t="s">
         <v>1050</v>
       </c>
-      <c r="D20" s="70"/>
-      <c r="E20" s="70"/>
+      <c r="D20" s="72"/>
+      <c r="E20" s="72"/>
       <c r="F20" s="68"/>
       <c r="G20" s="66"/>
       <c r="H20" s="66"/>
       <c r="I20" s="66"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="76"/>
+      <c r="A21" s="75"/>
       <c r="B21" s="42" t="s">
         <v>1051</v>
       </c>
-      <c r="C21" s="70" t="s">
+      <c r="C21" s="72" t="s">
         <v>1052</v>
       </c>
-      <c r="D21" s="70"/>
-      <c r="E21" s="70"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="72"/>
       <c r="F21" s="68"/>
       <c r="G21" s="66"/>
       <c r="H21" s="66"/>
       <c r="I21" s="66"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="76"/>
+      <c r="A22" s="75"/>
       <c r="B22" s="42" t="s">
         <v>1053</v>
       </c>
-      <c r="C22" s="70" t="s">
+      <c r="C22" s="72" t="s">
         <v>1054</v>
       </c>
-      <c r="D22" s="70"/>
-      <c r="E22" s="70"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="72"/>
       <c r="F22" s="68"/>
       <c r="G22" s="66"/>
       <c r="H22" s="66"/>
       <c r="I22" s="66"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="76"/>
+      <c r="A23" s="75"/>
       <c r="B23" s="42" t="s">
         <v>1055</v>
       </c>
-      <c r="C23" s="70" t="s">
+      <c r="C23" s="72" t="s">
         <v>1056</v>
       </c>
-      <c r="D23" s="70"/>
-      <c r="E23" s="70"/>
+      <c r="D23" s="72"/>
+      <c r="E23" s="72"/>
       <c r="F23" s="68"/>
       <c r="G23" s="66"/>
       <c r="H23" s="66"/>
       <c r="I23" s="66"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="76" t="s">
+      <c r="A24" s="75" t="s">
         <v>1057</v>
       </c>
       <c r="B24" s="42" t="s">
         <v>1049</v>
       </c>
-      <c r="C24" s="70" t="s">
+      <c r="C24" s="72" t="s">
         <v>1058</v>
       </c>
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="72"/>
       <c r="F24" s="68"/>
       <c r="G24" s="66"/>
       <c r="H24" s="66"/>
       <c r="I24" s="66"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="76"/>
+      <c r="A25" s="75"/>
       <c r="B25" s="42" t="s">
         <v>1059</v>
       </c>
-      <c r="C25" s="70" t="s">
+      <c r="C25" s="72" t="s">
         <v>1060</v>
       </c>
-      <c r="D25" s="70"/>
-      <c r="E25" s="70"/>
+      <c r="D25" s="72"/>
+      <c r="E25" s="72"/>
       <c r="F25" s="68"/>
       <c r="G25" s="66"/>
       <c r="H25" s="66"/>
       <c r="I25" s="66"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="76"/>
+      <c r="A26" s="75"/>
       <c r="B26" s="42" t="s">
         <v>1053</v>
       </c>
-      <c r="C26" s="70" t="s">
+      <c r="C26" s="72" t="s">
         <v>1061</v>
       </c>
-      <c r="D26" s="70"/>
-      <c r="E26" s="70"/>
+      <c r="D26" s="72"/>
+      <c r="E26" s="72"/>
       <c r="F26" s="68"/>
       <c r="G26" s="66"/>
       <c r="H26" s="66"/>
       <c r="I26" s="66"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="76"/>
+      <c r="A27" s="75"/>
       <c r="B27" s="42" t="s">
         <v>1055</v>
       </c>
-      <c r="C27" s="74" t="s">
+      <c r="C27" s="76" t="s">
         <v>1062</v>
       </c>
-      <c r="D27" s="74"/>
-      <c r="E27" s="74"/>
+      <c r="D27" s="76"/>
+      <c r="E27" s="76"/>
       <c r="F27" s="68"/>
       <c r="G27" s="66"/>
       <c r="H27" s="66"/>
@@ -27338,137 +27354,137 @@
       <c r="B28" s="45" t="s">
         <v>1064</v>
       </c>
-      <c r="C28" s="74" t="s">
+      <c r="C28" s="76" t="s">
         <v>1065</v>
       </c>
-      <c r="D28" s="74"/>
-      <c r="E28" s="74"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
       <c r="F28" s="68"/>
       <c r="G28" s="66"/>
       <c r="H28" s="66"/>
       <c r="I28" s="66"/>
     </row>
     <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="76" t="s">
+      <c r="A29" s="75" t="s">
         <v>1066</v>
       </c>
       <c r="B29" s="45" t="s">
         <v>1067</v>
       </c>
-      <c r="C29" s="74" t="s">
+      <c r="C29" s="76" t="s">
         <v>1068</v>
       </c>
-      <c r="D29" s="74"/>
-      <c r="E29" s="74"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
       <c r="F29" s="68"/>
       <c r="G29" s="66"/>
       <c r="H29" s="66"/>
       <c r="I29" s="66"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="76"/>
+      <c r="A30" s="75"/>
       <c r="B30" s="45" t="s">
         <v>1069</v>
       </c>
-      <c r="C30" s="74" t="s">
+      <c r="C30" s="76" t="s">
         <v>1070</v>
       </c>
-      <c r="D30" s="74"/>
-      <c r="E30" s="74"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="76"/>
       <c r="F30" s="68"/>
       <c r="G30" s="66"/>
       <c r="H30" s="66"/>
       <c r="I30" s="66"/>
     </row>
     <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="76" t="s">
+      <c r="A31" s="75" t="s">
         <v>1071</v>
       </c>
       <c r="B31" s="45" t="s">
         <v>1072</v>
       </c>
-      <c r="C31" s="74" t="s">
+      <c r="C31" s="76" t="s">
         <v>1073</v>
       </c>
-      <c r="D31" s="74"/>
-      <c r="E31" s="74"/>
+      <c r="D31" s="76"/>
+      <c r="E31" s="76"/>
       <c r="F31" s="68"/>
       <c r="G31" s="66"/>
       <c r="H31" s="66"/>
       <c r="I31" s="66"/>
     </row>
     <row r="32" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="76"/>
+      <c r="A32" s="75"/>
       <c r="B32" s="45" t="s">
         <v>1074</v>
       </c>
-      <c r="C32" s="74" t="s">
+      <c r="C32" s="76" t="s">
         <v>1075</v>
       </c>
-      <c r="D32" s="74"/>
-      <c r="E32" s="74"/>
+      <c r="D32" s="76"/>
+      <c r="E32" s="76"/>
       <c r="F32" s="68"/>
       <c r="G32" s="66"/>
       <c r="H32" s="66"/>
       <c r="I32" s="66"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="76" t="s">
+      <c r="A33" s="75" t="s">
         <v>1076</v>
       </c>
       <c r="B33" s="45" t="s">
         <v>1049</v>
       </c>
-      <c r="C33" s="74" t="s">
+      <c r="C33" s="76" t="s">
         <v>1077</v>
       </c>
-      <c r="D33" s="74"/>
-      <c r="E33" s="74"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
       <c r="F33" s="68"/>
       <c r="G33" s="66"/>
       <c r="H33" s="66"/>
       <c r="I33" s="66"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="76"/>
+      <c r="A34" s="75"/>
       <c r="B34" s="45" t="s">
         <v>1078</v>
       </c>
-      <c r="C34" s="74" t="s">
+      <c r="C34" s="76" t="s">
         <v>1079</v>
       </c>
-      <c r="D34" s="74"/>
-      <c r="E34" s="74"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
       <c r="F34" s="68"/>
       <c r="G34" s="66"/>
       <c r="H34" s="66"/>
       <c r="I34" s="66"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="76"/>
+      <c r="A35" s="75"/>
       <c r="B35" s="45" t="s">
         <v>1080</v>
       </c>
-      <c r="C35" s="74" t="s">
+      <c r="C35" s="76" t="s">
         <v>1081</v>
       </c>
-      <c r="D35" s="74"/>
-      <c r="E35" s="74"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
       <c r="F35" s="68"/>
       <c r="G35" s="66"/>
       <c r="H35" s="66"/>
       <c r="I35" s="66"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="76"/>
+      <c r="A36" s="75"/>
       <c r="B36" s="45" t="s">
         <v>151</v>
       </c>
-      <c r="C36" s="74" t="s">
+      <c r="C36" s="76" t="s">
         <v>1082</v>
       </c>
-      <c r="D36" s="74"/>
-      <c r="E36" s="74"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
       <c r="F36" s="68"/>
       <c r="G36" s="66"/>
       <c r="H36" s="66"/>
@@ -27481,97 +27497,97 @@
       <c r="B37" s="45" t="s">
         <v>1064</v>
       </c>
-      <c r="C37" s="74" t="s">
+      <c r="C37" s="76" t="s">
         <v>1084</v>
       </c>
-      <c r="D37" s="74"/>
-      <c r="E37" s="74"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
       <c r="F37" s="68"/>
       <c r="G37" s="66"/>
       <c r="H37" s="66"/>
       <c r="I37" s="66"/>
     </row>
     <row r="38" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="76" t="s">
+      <c r="A38" s="75" t="s">
         <v>1085</v>
       </c>
       <c r="B38" s="45" t="s">
         <v>1086</v>
       </c>
-      <c r="C38" s="74" t="s">
+      <c r="C38" s="76" t="s">
         <v>1087</v>
       </c>
-      <c r="D38" s="74"/>
-      <c r="E38" s="74"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
       <c r="F38" s="68"/>
       <c r="G38" s="66"/>
       <c r="H38" s="66"/>
       <c r="I38" s="66"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="76"/>
+      <c r="A39" s="75"/>
       <c r="B39" s="45" t="s">
         <v>1088</v>
       </c>
-      <c r="C39" s="74" t="s">
+      <c r="C39" s="76" t="s">
         <v>1089</v>
       </c>
-      <c r="D39" s="74"/>
-      <c r="E39" s="74"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
       <c r="F39" s="68"/>
       <c r="G39" s="66"/>
       <c r="H39" s="66"/>
       <c r="I39" s="66"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="76"/>
+      <c r="A40" s="75"/>
       <c r="B40" s="45" t="s">
         <v>1090</v>
       </c>
-      <c r="C40" s="74" t="s">
+      <c r="C40" s="76" t="s">
         <v>1091</v>
       </c>
-      <c r="D40" s="74"/>
-      <c r="E40" s="74"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
       <c r="F40" s="68"/>
       <c r="G40" s="66"/>
       <c r="H40" s="66"/>
       <c r="I40" s="66"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="76" t="s">
+      <c r="A41" s="75" t="s">
         <v>1092</v>
       </c>
       <c r="B41" s="45" t="s">
         <v>1093</v>
       </c>
-      <c r="C41" s="74" t="s">
+      <c r="C41" s="76" t="s">
         <v>1094</v>
       </c>
-      <c r="D41" s="74"/>
-      <c r="E41" s="74"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
       <c r="F41" s="68"/>
       <c r="G41" s="66"/>
       <c r="H41" s="66"/>
       <c r="I41" s="66"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="76"/>
+      <c r="A42" s="75"/>
       <c r="B42" s="45" t="s">
         <v>1095</v>
       </c>
-      <c r="C42" s="74" t="s">
+      <c r="C42" s="76" t="s">
         <v>1096</v>
       </c>
-      <c r="D42" s="74"/>
-      <c r="E42" s="74"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
       <c r="F42" s="68"/>
       <c r="G42" s="66"/>
       <c r="H42" s="66"/>
       <c r="I42" s="66"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="76"/>
+      <c r="A43" s="75"/>
       <c r="B43" s="45" t="s">
         <v>1097</v>
       </c>
@@ -27586,47 +27602,47 @@
       <c r="I43" s="66"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="76"/>
+      <c r="A44" s="75"/>
       <c r="B44" s="45" t="s">
         <v>1099</v>
       </c>
-      <c r="C44" s="75" t="s">
+      <c r="C44" s="74" t="s">
         <v>1100</v>
       </c>
-      <c r="D44" s="75"/>
-      <c r="E44" s="75"/>
+      <c r="D44" s="74"/>
+      <c r="E44" s="74"/>
       <c r="F44" s="68"/>
       <c r="G44" s="66"/>
       <c r="H44" s="66"/>
       <c r="I44" s="66"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="76" t="s">
+      <c r="A45" s="75" t="s">
         <v>1101</v>
       </c>
       <c r="B45" s="45" t="s">
         <v>1102</v>
       </c>
-      <c r="C45" s="75" t="s">
+      <c r="C45" s="74" t="s">
         <v>1103</v>
       </c>
-      <c r="D45" s="75"/>
-      <c r="E45" s="75"/>
+      <c r="D45" s="74"/>
+      <c r="E45" s="74"/>
       <c r="F45" s="68"/>
       <c r="G45" s="66"/>
       <c r="H45" s="66"/>
       <c r="I45" s="66"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="76"/>
+      <c r="A46" s="75"/>
       <c r="B46" s="45" t="s">
         <v>1104</v>
       </c>
-      <c r="C46" s="75" t="s">
+      <c r="C46" s="74" t="s">
         <v>1105</v>
       </c>
-      <c r="D46" s="75"/>
-      <c r="E46" s="75"/>
+      <c r="D46" s="74"/>
+      <c r="E46" s="74"/>
       <c r="F46" s="68"/>
       <c r="G46" s="66"/>
       <c r="H46" s="66"/>
@@ -27639,11 +27655,11 @@
       <c r="B47" s="45" t="s">
         <v>1064</v>
       </c>
-      <c r="C47" s="75" t="s">
+      <c r="C47" s="74" t="s">
         <v>1107</v>
       </c>
-      <c r="D47" s="75"/>
-      <c r="E47" s="75"/>
+      <c r="D47" s="74"/>
+      <c r="E47" s="74"/>
       <c r="F47" s="68"/>
       <c r="G47" s="66"/>
       <c r="H47" s="66"/>
@@ -27656,165 +27672,165 @@
       <c r="B48" s="45" t="s">
         <v>1109</v>
       </c>
-      <c r="C48" s="75" t="s">
+      <c r="C48" s="74" t="s">
         <v>1110</v>
       </c>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
+      <c r="D48" s="74"/>
+      <c r="E48" s="74"/>
       <c r="F48" s="68"/>
       <c r="G48" s="66"/>
       <c r="H48" s="66"/>
       <c r="I48" s="66"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="76" t="s">
+      <c r="A49" s="75" t="s">
         <v>1111</v>
       </c>
       <c r="B49" s="45" t="s">
         <v>1112</v>
       </c>
-      <c r="C49" s="75" t="s">
+      <c r="C49" s="74" t="s">
         <v>1113</v>
       </c>
-      <c r="D49" s="75"/>
-      <c r="E49" s="75"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="74"/>
       <c r="F49" s="68"/>
       <c r="G49" s="66"/>
       <c r="H49" s="66"/>
       <c r="I49" s="66"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="76"/>
+      <c r="A50" s="75"/>
       <c r="B50" s="45" t="s">
         <v>1114</v>
       </c>
-      <c r="C50" s="75" t="s">
+      <c r="C50" s="74" t="s">
         <v>1115</v>
       </c>
-      <c r="D50" s="75"/>
-      <c r="E50" s="75"/>
+      <c r="D50" s="74"/>
+      <c r="E50" s="74"/>
       <c r="F50" s="68"/>
       <c r="G50" s="66"/>
       <c r="H50" s="66"/>
       <c r="I50" s="66"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="76"/>
+      <c r="A51" s="75"/>
       <c r="B51" s="45" t="s">
         <v>1059</v>
       </c>
-      <c r="C51" s="75" t="s">
+      <c r="C51" s="74" t="s">
         <v>1116</v>
       </c>
-      <c r="D51" s="75"/>
-      <c r="E51" s="75"/>
+      <c r="D51" s="74"/>
+      <c r="E51" s="74"/>
       <c r="F51" s="68"/>
       <c r="G51" s="66"/>
       <c r="H51" s="66"/>
       <c r="I51" s="66"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="76"/>
+      <c r="A52" s="75"/>
       <c r="B52" s="45" t="s">
         <v>1117</v>
       </c>
-      <c r="C52" s="75" t="s">
+      <c r="C52" s="74" t="s">
         <v>1118</v>
       </c>
-      <c r="D52" s="75"/>
-      <c r="E52" s="75"/>
+      <c r="D52" s="74"/>
+      <c r="E52" s="74"/>
       <c r="F52" s="68"/>
       <c r="G52" s="66"/>
       <c r="H52" s="66"/>
       <c r="I52" s="66"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" s="76"/>
+      <c r="A53" s="75"/>
       <c r="B53" s="45" t="s">
         <v>1055</v>
       </c>
-      <c r="C53" s="75" t="s">
+      <c r="C53" s="74" t="s">
         <v>1119</v>
       </c>
-      <c r="D53" s="75"/>
-      <c r="E53" s="75"/>
+      <c r="D53" s="74"/>
+      <c r="E53" s="74"/>
       <c r="F53" s="68"/>
       <c r="G53" s="66"/>
       <c r="H53" s="66"/>
       <c r="I53" s="66"/>
     </row>
     <row r="54" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="76" t="s">
+      <c r="A54" s="75" t="s">
         <v>1120</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>1121</v>
       </c>
-      <c r="C54" s="75" t="s">
+      <c r="C54" s="74" t="s">
         <v>1122</v>
       </c>
-      <c r="D54" s="75"/>
-      <c r="E54" s="75"/>
+      <c r="D54" s="74"/>
+      <c r="E54" s="74"/>
       <c r="F54" s="68"/>
       <c r="G54" s="66"/>
       <c r="H54" s="66"/>
       <c r="I54" s="66"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="76"/>
+      <c r="A55" s="75"/>
       <c r="B55" s="5" t="s">
         <v>1123</v>
       </c>
-      <c r="C55" s="75" t="s">
+      <c r="C55" s="74" t="s">
         <v>1124</v>
       </c>
-      <c r="D55" s="75"/>
-      <c r="E55" s="75"/>
+      <c r="D55" s="74"/>
+      <c r="E55" s="74"/>
       <c r="F55" s="68"/>
       <c r="G55" s="66"/>
       <c r="H55" s="66"/>
       <c r="I55" s="66"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="76"/>
+      <c r="A56" s="75"/>
       <c r="B56" s="5" t="s">
         <v>1125</v>
       </c>
-      <c r="C56" s="75" t="s">
+      <c r="C56" s="74" t="s">
         <v>1126</v>
       </c>
-      <c r="D56" s="75"/>
-      <c r="E56" s="75"/>
+      <c r="D56" s="74"/>
+      <c r="E56" s="74"/>
       <c r="F56" s="68"/>
       <c r="G56" s="66"/>
       <c r="H56" s="66"/>
       <c r="I56" s="66"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="76"/>
+      <c r="A57" s="75"/>
       <c r="B57" s="5" t="s">
         <v>1127</v>
       </c>
-      <c r="C57" s="75" t="s">
+      <c r="C57" s="74" t="s">
         <v>1128</v>
       </c>
-      <c r="D57" s="75"/>
-      <c r="E57" s="75"/>
+      <c r="D57" s="74"/>
+      <c r="E57" s="74"/>
       <c r="F57" s="68"/>
       <c r="G57" s="66"/>
       <c r="H57" s="66"/>
       <c r="I57" s="66"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="76"/>
+      <c r="A58" s="75"/>
       <c r="B58" s="5" t="s">
         <v>1129</v>
       </c>
-      <c r="C58" s="75" t="s">
+      <c r="C58" s="74" t="s">
         <v>1130</v>
       </c>
-      <c r="D58" s="75"/>
-      <c r="E58" s="75"/>
+      <c r="D58" s="74"/>
+      <c r="E58" s="74"/>
       <c r="F58" s="68"/>
       <c r="G58" s="66"/>
       <c r="H58" s="66"/>
@@ -27827,88 +27843,88 @@
       <c r="B59" s="5" t="s">
         <v>1064</v>
       </c>
-      <c r="C59" s="75" t="s">
+      <c r="C59" s="74" t="s">
         <v>1132</v>
       </c>
-      <c r="D59" s="75"/>
-      <c r="E59" s="75"/>
+      <c r="D59" s="74"/>
+      <c r="E59" s="74"/>
       <c r="F59" s="68"/>
       <c r="G59" s="66"/>
       <c r="H59" s="66"/>
       <c r="I59" s="66"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="76" t="s">
+      <c r="A60" s="75" t="s">
         <v>1133</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>1134</v>
       </c>
-      <c r="C60" s="75" t="s">
+      <c r="C60" s="74" t="s">
         <v>1135</v>
       </c>
-      <c r="D60" s="75"/>
-      <c r="E60" s="75"/>
+      <c r="D60" s="74"/>
+      <c r="E60" s="74"/>
       <c r="F60" s="68"/>
       <c r="G60" s="66"/>
       <c r="H60" s="66"/>
       <c r="I60" s="66"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="76"/>
+      <c r="A61" s="75"/>
       <c r="B61" s="5" t="s">
         <v>1136</v>
       </c>
-      <c r="C61" s="75" t="s">
+      <c r="C61" s="74" t="s">
         <v>1137</v>
       </c>
-      <c r="D61" s="75"/>
-      <c r="E61" s="75"/>
+      <c r="D61" s="74"/>
+      <c r="E61" s="74"/>
       <c r="F61" s="68"/>
       <c r="G61" s="66"/>
       <c r="H61" s="66"/>
       <c r="I61" s="66"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="76"/>
+      <c r="A62" s="75"/>
       <c r="B62" s="5" t="s">
         <v>1138</v>
       </c>
-      <c r="C62" s="75" t="s">
+      <c r="C62" s="74" t="s">
         <v>1139</v>
       </c>
-      <c r="D62" s="75"/>
-      <c r="E62" s="75"/>
+      <c r="D62" s="74"/>
+      <c r="E62" s="74"/>
       <c r="F62" s="68"/>
       <c r="G62" s="66"/>
       <c r="H62" s="66"/>
       <c r="I62" s="66"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="76"/>
+      <c r="A63" s="75"/>
       <c r="B63" s="5" t="s">
         <v>1140</v>
       </c>
-      <c r="C63" s="75" t="s">
+      <c r="C63" s="74" t="s">
         <v>1141</v>
       </c>
-      <c r="D63" s="75"/>
-      <c r="E63" s="75"/>
+      <c r="D63" s="74"/>
+      <c r="E63" s="74"/>
       <c r="F63" s="68"/>
       <c r="G63" s="66"/>
       <c r="H63" s="66"/>
       <c r="I63" s="66"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A64" s="76"/>
+      <c r="A64" s="75"/>
       <c r="B64" s="5" t="s">
         <v>1142</v>
       </c>
-      <c r="C64" s="75" t="s">
+      <c r="C64" s="74" t="s">
         <v>1143</v>
       </c>
-      <c r="D64" s="75"/>
-      <c r="E64" s="75"/>
+      <c r="D64" s="74"/>
+      <c r="E64" s="74"/>
       <c r="F64" s="68"/>
       <c r="G64" s="66"/>
       <c r="H64" s="66"/>
@@ -27916,36 +27932,66 @@
     </row>
   </sheetData>
   <mergeCells count="114">
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="F62:I62"/>
-    <mergeCell ref="F63:I63"/>
-    <mergeCell ref="F64:I64"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F38:I38"/>
-    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="F29:I29"/>
     <mergeCell ref="C63:E63"/>
     <mergeCell ref="C64:E64"/>
     <mergeCell ref="A54:A58"/>
@@ -27970,66 +28016,36 @@
     <mergeCell ref="A45:A46"/>
     <mergeCell ref="C52:E52"/>
     <mergeCell ref="C53:E53"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="A15:A19"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -28501,6 +28517,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C13:F13"/>
@@ -28517,9 +28536,6 @@
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C29:F29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -29290,6 +29306,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="F18:I18"/>
     <mergeCell ref="F17:I17"/>
@@ -29302,13 +29325,6 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -29674,6 +29690,18 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="F12:I12"/>
     <mergeCell ref="F9:I9"/>
@@ -29681,18 +29709,6 @@
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="F11:I11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -30154,19 +30170,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:I14"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="F22:I22"/>
     <mergeCell ref="F23:I23"/>
@@ -30180,6 +30183,19 @@
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="F10:I10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -31151,29 +31167,33 @@
     </row>
   </sheetData>
   <mergeCells count="63">
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="F35:I35"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="F32:I32"/>
     <mergeCell ref="C24:D24"/>
@@ -31187,33 +31207,29 @@
     <mergeCell ref="F30:I30"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="F31:I31"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="F60:I60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -31693,13 +31709,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:I15"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C20:D20"/>
@@ -31710,6 +31719,13 @@
     <mergeCell ref="F18:I18"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="F19:I19"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:I15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -32112,6 +32128,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="C20:D20"/>
@@ -32124,11 +32145,6 @@
     <mergeCell ref="F20:I20"/>
     <mergeCell ref="F17:I17"/>
     <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -32160,26 +32176,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="eda01c43-580c-44af-a5fd-4ea1802e476c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004592A3ADBB772D4689FCD56C8516F45D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e6dee92c918a6173969cc6829137ba01">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c" xmlns:ns3="eda01c43-580c-44af-a5fd-4ea1802e476c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2e0be94b10bd652582aed8d62fec2d74" ns2:_="" ns3:_="">
     <xsd:import namespace="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c"/>
@@ -32408,10 +32404,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="eda01c43-580c-44af-a5fd-4ea1802e476c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB40FF6F-009E-4D48-B4D3-33D1A3C62497}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA0A127A-D0D0-4182-84ED-7D64B945D928}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c"/>
+    <ds:schemaRef ds:uri="eda01c43-580c-44af-a5fd-4ea1802e476c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -32434,20 +32461,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA0A127A-D0D0-4182-84ED-7D64B945D928}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB40FF6F-009E-4D48-B4D3-33D1A3C62497}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9a1da51d-87f1-4c78-b9e6-a6488d1ad35c"/>
-    <ds:schemaRef ds:uri="eda01c43-580c-44af-a5fd-4ea1802e476c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
✨ add invasive mean bp code to vital signs value set
</commit_message>
<xml_diff>
--- a/CommonDataModel.xlsx
+++ b/CommonDataModel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\db\dt4h\common-data-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAC1BCF-B7D7-4289-BB41-6339F2BD48B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418003E4-1E73-49B3-855F-E5FAFB2CB239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="10635" windowWidth="38640" windowHeight="21120" tabRatio="901" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" tabRatio="901" firstSheet="8" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="10" r:id="rId1"/>
@@ -864,7 +864,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4696" uniqueCount="2026">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4701" uniqueCount="2028">
   <si>
     <t>Required</t>
   </si>
@@ -6962,6 +6962,12 @@
   </si>
   <si>
     <t>Passive smoker</t>
+  </si>
+  <si>
+    <t>76214-6</t>
+  </si>
+  <si>
+    <t>Invasive Mean blood pressure</t>
   </si>
 </sst>
 </file>
@@ -7228,7 +7234,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -7358,6 +7364,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53"/>
@@ -11704,7 +11711,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0672E625-A39D-44D8-824F-D75CA3AC11CE}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.33203125" customWidth="1"/>
@@ -12292,42 +12299,42 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>1354</v>
+        <v>2027</v>
       </c>
       <c r="B31" t="s">
-        <v>1355</v>
+        <v>2026</v>
       </c>
       <c r="C31" s="65" t="s">
         <v>345</v>
       </c>
       <c r="D31" s="65"/>
       <c r="E31" s="33" t="s">
-        <v>667</v>
-      </c>
-      <c r="F31" t="s">
-        <v>1808</v>
-      </c>
-      <c r="G31" s="66"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="66"/>
+        <v>1350</v>
+      </c>
+      <c r="F31" s="77" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="49" t="s">
-        <v>1686</v>
-      </c>
-      <c r="B32" s="49" t="s">
-        <v>1687</v>
+      <c r="A32" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1355</v>
       </c>
       <c r="C32" s="65" t="s">
         <v>345</v>
       </c>
       <c r="D32" s="65"/>
       <c r="E32" s="33" t="s">
-        <v>1350</v>
+        <v>667</v>
       </c>
       <c r="F32" t="s">
-        <v>1809</v>
+        <v>1808</v>
       </c>
       <c r="G32" s="66"/>
       <c r="H32" s="66"/>
@@ -12336,10 +12343,10 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="49" t="s">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="B33" s="49" t="s">
-        <v>1689</v>
+        <v>1687</v>
       </c>
       <c r="C33" s="65" t="s">
         <v>345</v>
@@ -12358,10 +12365,10 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="49" t="s">
-        <v>1690</v>
+        <v>1688</v>
       </c>
       <c r="B34" s="49" t="s">
-        <v>1691</v>
+        <v>1689</v>
       </c>
       <c r="C34" s="65" t="s">
         <v>345</v>
@@ -12380,16 +12387,16 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="49" t="s">
-        <v>1778</v>
+        <v>1690</v>
       </c>
       <c r="B35" s="49" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="C35" s="65" t="s">
         <v>345</v>
       </c>
       <c r="D35" s="65"/>
-      <c r="E35" s="56" t="s">
+      <c r="E35" s="33" t="s">
         <v>1350</v>
       </c>
       <c r="F35" t="s">
@@ -12401,37 +12408,59 @@
       <c r="J35" s="66"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>1844</v>
-      </c>
-      <c r="B36" t="s">
-        <v>1845</v>
+      <c r="A36" s="49" t="s">
+        <v>1778</v>
+      </c>
+      <c r="B36" s="49" t="s">
+        <v>1692</v>
       </c>
       <c r="C36" s="65" t="s">
         <v>345</v>
       </c>
       <c r="D36" s="65"/>
-      <c r="E36" t="s">
-        <v>1846</v>
-      </c>
+      <c r="E36" s="56" t="s">
+        <v>1350</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G36" s="66"/>
+      <c r="H36" s="66"/>
+      <c r="I36" s="66"/>
+      <c r="J36" s="66"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1848</v>
+        <v>1844</v>
       </c>
       <c r="B37" t="s">
-        <v>1847</v>
+        <v>1845</v>
       </c>
       <c r="C37" s="65" t="s">
         <v>345</v>
       </c>
       <c r="D37" s="65"/>
       <c r="E37" t="s">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1847</v>
+      </c>
+      <c r="C38" s="65" t="s">
+        <v>345</v>
+      </c>
+      <c r="D38" s="65"/>
+      <c r="E38" t="s">
         <v>667</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="49">
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="C21:D21"/>
@@ -12455,9 +12484,9 @@
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="G33:J33"/>
     <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="G29:J29"/>
@@ -12466,20 +12495,21 @@
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
-    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="C31:D31"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G23:J23"/>
     <mergeCell ref="G24:J24"/>
     <mergeCell ref="G25:J25"/>
     <mergeCell ref="G26:J26"/>
-    <mergeCell ref="C36:D36"/>
     <mergeCell ref="C37:D37"/>
-    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="C38:D38"/>
     <mergeCell ref="G34:J34"/>
     <mergeCell ref="G35:J35"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
     <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C33:D33"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E13:F21" xr:uid="{7FAB08B6-9907-44B4-A82A-4A3E200D36A8}">
@@ -28522,11 +28552,6 @@
     <mergeCell ref="C29:F29"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C17:F17"/>
     <mergeCell ref="C30:F30"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="C20:F20"/>
@@ -28536,6 +28561,11 @@
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C17:F17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>